<commit_message>
Update StickerBinStickersCosts v2.xlsx with revised cost data
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A21E20-3BAA-4ACF-A3E6-A31FEB4D9FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED96A0C-EAFE-4268-9582-A79529B7C103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="199">
   <si>
     <t>Tier 1 Equipment Costs — Sticker Side Hustle</t>
   </si>
@@ -160,31 +160,13 @@
     <t>R&amp;D / Testing Materials (one-off, sunk cost — see Bin-Sticker-Material-Test-Plan.md)</t>
   </si>
   <si>
-    <t>Test vinyl &amp; laminate samples (Cricut vs Stickiply, Tests 1–5)</t>
-  </si>
-  <si>
     <t>R&amp;D</t>
   </si>
   <si>
-    <t>Cost of vinyl/laminate sheets consumed making comparison samples — separate from the per-pack production materials costed in the Bin Stickers sheet. See Bin-Sticker-Material-Test-Plan.md.</t>
-  </si>
-  <si>
-    <t>Test packaging materials (Test 6 — envelopes, tissue, padded mailers, boxes)</t>
-  </si>
-  <si>
     <t>One-off purchase of all 4 packaging candidates for side-by-side comparison. See Bin-Sticker-Shipping-Plan.md 'Testing shopping list' (~£33–35 total as pinned there — update once actually spent).</t>
   </si>
   <si>
-    <t>Test postage (post-to-self trials)</t>
-  </si>
-  <si>
     <t>2nd Class postage for the 4 test parcels in Test 6. See Bin-Sticker-Shipping-Plan.md.</t>
-  </si>
-  <si>
-    <t>Corner punch / cutter verification samples (offcut vinyl+laminate)</t>
-  </si>
-  <si>
-    <t>See Material Test Plan addendum (July 2026) — corner punch &amp; peel-nick verification on laminated vinyl.</t>
   </si>
   <si>
     <t>R&amp;D SUBTOTAL</t>
@@ -615,6 +597,57 @@
   <si>
     <t>Self-Healing Cutting Mat (A4)</t>
   </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>Matte Self-Adhesive Laminate | Pro UV × 1</t>
+  </si>
+  <si>
+    <t>Printable Vinyl Sticker Paper | Clear (A4) × 1</t>
+  </si>
+  <si>
+    <t>Printable Vinyl Sticker Paper | Glossy (A4) × 1</t>
+  </si>
+  <si>
+    <t>Brown Kraft Card, A4 Card 250GSM Thick Kraft Card Stock for Cards Making, Scrapbook, Office Printing and Arts or Crafts DIY (25 Sheets)</t>
+  </si>
+  <si>
+    <t>Double Dragon 50-Pack A6 C6 Manilla Hard Board Backed Envelopes | 162mm x 114mm | 'Please Do Not Bend' Printed | Padded &amp; Tamper-Proof | Self-Seal Closure</t>
+  </si>
+  <si>
+    <t>White Card, A4 Card 250GSM Thick Card Stock for Cards Making, Scrapbook, Office Printing and Arts or Crafts DIY (25 Sheets)</t>
+  </si>
+  <si>
+    <t>SmithPackaging A4 Self Adhesive Address Labels, 1 Label Per Sheet, 100 Sheets, 199.6 x 289.1mm, 100 Labels</t>
+  </si>
+  <si>
+    <t>40 Sheets of Acid Free Tissue Paper Cool White MG 17gsm Clothing Storage Gift Wrapping Decorative Sketch and Cutting Large Tissue Paper for Art Craft and Packing - 500mm x 750mm</t>
+  </si>
+  <si>
+    <t>Triplast White Bubble Padded Envelopes - Pick Qty &amp; Size: 10 x 1/A (100x165mm) A6 Envelopes - Large Letter Postal Bags with Bubble Wrap Lining and Peel &amp; Seal Strip for Royal Mail Shipping &amp; Postage</t>
+  </si>
+  <si>
+    <t>AKAR White A6/C6 Large Letter Postal Box - 112x163x20 mm - Letterbox Pip Royal Mail Small Boxes for Posting [Pack of 50]</t>
+  </si>
+  <si>
+    <t>amazon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stickiply </t>
+  </si>
+  <si>
+    <t>Printable Waterproof Sticker Set – A4 (20 ct), White</t>
+  </si>
+  <si>
+    <t>Printable Waterproof Sticker Set – A4 (20 ct), Transparent</t>
+  </si>
+  <si>
+    <t>Shipping</t>
+  </si>
+  <si>
+    <t>cricut</t>
+  </si>
 </sst>
 </file>
 
@@ -624,7 +657,7 @@
     <numFmt numFmtId="164" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -789,6 +822,20 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF555555"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -840,16 +887,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -889,12 +936,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="19" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -903,8 +948,14 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1167,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -1181,100 +1232,100 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>370</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>0</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>0</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>105</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="51" t="s">
-        <v>186</v>
+      <c r="E8" s="48" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <v>0</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1297,7 +1348,7 @@
         <v>19</v>
       </c>
       <c r="B11">
-        <v>4.49</v>
+        <v>7</v>
       </c>
       <c r="C11" t="s">
         <v>7</v>
@@ -1321,320 +1372,536 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="52" t="s">
-        <v>187</v>
+      <c r="A13" s="49" t="s">
+        <v>181</v>
       </c>
       <c r="B13">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <f>SUM(B5:B13)</f>
-        <v>526.49</v>
-      </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
+        <v>529</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="7">
         <v>96</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="7">
         <v>249.99</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="7">
         <v>11.19</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="7">
         <v>250</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <f>SUM(B18:B21)</f>
         <v>607.18000000000006</v>
       </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-    </row>
-    <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="14">
         <f>B14+B18</f>
-        <v>622.49</v>
-      </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D30" s="16" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="18" t="s">
+      <c r="E30" s="16" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.35">
+      <c r="A31" s="53" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" s="18">
+        <v>13</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="1"/>
+      <c r="E31">
+        <v>25</v>
+      </c>
+      <c r="F31">
+        <f>B31/E31</f>
+        <v>0.52</v>
+      </c>
+      <c r="G31" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.35">
+      <c r="A32" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="B32" s="18">
+        <v>8</v>
+      </c>
+      <c r="C32" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="19">
-        <v>0</v>
-      </c>
-      <c r="C31" s="18" t="s">
+      <c r="D32" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E32">
+        <v>10</v>
+      </c>
+      <c r="F32">
+        <f t="shared" ref="F32:F42" si="0">B32/E32</f>
+        <v>0.8</v>
+      </c>
+      <c r="G32" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+      <c r="A33" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="B33" s="18">
+        <v>5.85</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="18" t="s">
+      <c r="E33">
+        <v>10</v>
+      </c>
+      <c r="F33">
+        <f t="shared" si="0"/>
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="G33" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="54" t="s">
+        <v>186</v>
+      </c>
+      <c r="B34" s="18">
+        <v>6</v>
+      </c>
+      <c r="C34" s="17"/>
+      <c r="D34" s="1"/>
+      <c r="E34">
+        <v>25</v>
+      </c>
+      <c r="F34">
+        <f t="shared" si="0"/>
+        <v>0.24</v>
+      </c>
+      <c r="G34" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="54" t="s">
+        <v>187</v>
+      </c>
+      <c r="B35" s="18">
+        <v>7.37</v>
+      </c>
+      <c r="C35" s="17"/>
+      <c r="D35" s="1"/>
+      <c r="E35">
+        <v>50</v>
+      </c>
+      <c r="F35">
+        <f t="shared" si="0"/>
+        <v>0.1474</v>
+      </c>
+      <c r="G35" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="54" t="s">
+        <v>188</v>
+      </c>
+      <c r="B36" s="18">
+        <v>6</v>
+      </c>
+      <c r="C36" s="17"/>
+      <c r="D36" s="1"/>
+      <c r="E36">
+        <v>25</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="0"/>
+        <v>0.24</v>
+      </c>
+      <c r="G36" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="54" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="18">
+        <v>9</v>
+      </c>
+      <c r="C37" s="17"/>
+      <c r="D37" s="1"/>
+      <c r="E37">
+        <v>100</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="0"/>
+        <v>0.09</v>
+      </c>
+      <c r="G37" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="54" t="s">
+        <v>190</v>
+      </c>
+      <c r="B38" s="18">
+        <v>5</v>
+      </c>
+      <c r="C38" s="17"/>
+      <c r="D38" s="1"/>
+      <c r="E38">
+        <v>40</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="0"/>
+        <v>0.125</v>
+      </c>
+      <c r="G38" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" s="54" t="s">
+        <v>191</v>
+      </c>
+      <c r="B39" s="18">
+        <v>6.09</v>
+      </c>
+      <c r="C39" s="17"/>
+      <c r="D39" s="1"/>
+      <c r="E39">
+        <v>10</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="0"/>
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="G39" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="54" t="s">
+        <v>192</v>
+      </c>
+      <c r="B40" s="18">
+        <v>10</v>
+      </c>
+      <c r="C40" s="17"/>
+      <c r="D40" s="1"/>
+      <c r="E40">
+        <v>50</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="0"/>
+        <v>0.2</v>
+      </c>
+      <c r="G40" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>195</v>
+      </c>
+      <c r="B41" s="18">
+        <v>13</v>
+      </c>
+      <c r="C41" s="17"/>
+      <c r="D41" s="1"/>
+      <c r="E41">
+        <v>20</v>
+      </c>
+      <c r="F41">
+        <f>(B41+I41)/E41</f>
+        <v>0.85</v>
+      </c>
+      <c r="G41" t="s">
+        <v>198</v>
+      </c>
+      <c r="H41" t="s">
+        <v>197</v>
+      </c>
+      <c r="I41">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>196</v>
+      </c>
+      <c r="B42" s="18">
+        <v>13</v>
+      </c>
+      <c r="C42" s="17"/>
+      <c r="D42" s="1"/>
+      <c r="E42">
+        <v>20</v>
+      </c>
+      <c r="F42">
+        <f>(B42+I42)/E42</f>
+        <v>0.85</v>
+      </c>
+      <c r="G42" t="s">
+        <v>198</v>
+      </c>
+      <c r="H42" t="s">
+        <v>197</v>
+      </c>
+      <c r="I42">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B32" s="19">
-        <v>0</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D32" s="5" t="s">
+      <c r="B43" s="20">
+        <f>SUM(B31:B42)</f>
+        <v>102.31</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="21" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="s">
+      <c r="B45" s="22">
+        <f>B14+B43</f>
+        <v>631.30999999999995</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="19">
-        <v>0</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" s="5" t="s">
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
+    </row>
+    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="23" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="18" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="19">
-        <v>0</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="5" t="s">
+      <c r="B49" s="50"/>
+      <c r="C49" s="50"/>
+      <c r="D49" s="50"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="17" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="20" t="s">
+      <c r="B51" s="18">
+        <v>6</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B35" s="21">
-        <f>SUM(B31:B34)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="22" t="s">
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="23">
-        <f>B14+B35</f>
-        <v>526.49</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-    </row>
-    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="24" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B43" s="19">
-        <v>6</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B44" s="25">
+      <c r="B52" s="24">
         <f>'Bin Stickers 100x150 4pk'!B68</f>
         <v>2.31</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B45" s="27">
-        <f>B43-B44</f>
+      <c r="D52" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="26">
+        <f>B51-B52</f>
         <v>3.69</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B47" s="28">
-        <f>B37</f>
-        <v>526.49</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="B48" s="29">
-        <f>IFERROR(B47/B45,"N/A")</f>
-        <v>142.68021680216802</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B49" s="29">
-        <f>IFERROR(B48*'Bin Stickers 100x150 4pk'!B7,"N/A")</f>
-        <v>570.72086720867208</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B55" s="27">
+        <f>B45</f>
+        <v>631.30999999999995</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="28">
+        <f>IFERROR(B55/B53,"N/A")</f>
+        <v>171.08672086720867</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" s="28">
+        <f>IFERROR(B56*'Bin Stickers 100x150 4pk'!B7,"N/A")</f>
+        <v>684.34688346883468</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="B59" s="50"/>
+      <c r="C59" s="50"/>
+      <c r="D59" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A59:D59"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A34" r:id="rId1" display="https://www.amazon.co.uk/dp/B0DK3V552G?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{A9C8AD4F-C0F2-4B99-B059-0E9F2D2424A2}"/>
+    <hyperlink ref="A35" r:id="rId2" display="https://www.amazon.co.uk/dp/B0DXY7Q984?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{AB31E489-0250-4669-97F2-EAF798F19B62}"/>
+    <hyperlink ref="A36" r:id="rId3" display="https://www.amazon.co.uk/dp/B0DJZFTP56?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{C948CAFA-9C08-4728-9912-18E8497EE6AE}"/>
+    <hyperlink ref="A37" r:id="rId4" display="https://www.amazon.co.uk/dp/B082WLC8BJ?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{72A31724-3B9B-4489-B08D-FE4A178541E1}"/>
+    <hyperlink ref="A38" r:id="rId5" display="https://www.amazon.co.uk/dp/B0BNQW8LY3?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{9811E86E-C503-4D1D-B2D2-F0C78911EB80}"/>
+    <hyperlink ref="A39" r:id="rId6" display="https://www.amazon.co.uk/dp/B0DFZ6585M?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{41981F4F-A3B7-41C8-A422-E74EF0BB9B1D}"/>
+    <hyperlink ref="A40" r:id="rId7" display="https://www.amazon.co.uk/dp/B094454Q6P?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{7DBA85D2-65A4-4DBA-9873-46396AB68A6E}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1651,256 +1918,256 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
-        <v>63</v>
+      <c r="A1" s="29" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
-        <v>64</v>
+      <c r="A2" s="30" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
-        <v>65</v>
+      <c r="A4" s="31" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="33" t="s">
+      <c r="B5" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>69</v>
+        <v>61</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="34">
+        <v>64</v>
+      </c>
+      <c r="B7" s="33">
         <v>4</v>
       </c>
-      <c r="C7" s="31" t="s">
-        <v>71</v>
+      <c r="C7" s="30" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="34">
+        <v>66</v>
+      </c>
+      <c r="B8" s="33">
         <v>1</v>
       </c>
-      <c r="C8" s="31" t="s">
-        <v>73</v>
+      <c r="C8" s="30" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="32" t="s">
-        <v>74</v>
+      <c r="A10" s="31" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="33" t="s">
+      <c r="B11" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="35">
+        <v>70</v>
+      </c>
+      <c r="B12" s="34">
         <v>0.4</v>
       </c>
-      <c r="C12" s="31" t="s">
-        <v>77</v>
+      <c r="C12" s="30" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>78</v>
-      </c>
-      <c r="B13" s="35">
+        <v>72</v>
+      </c>
+      <c r="B13" s="34">
         <v>0.2</v>
       </c>
-      <c r="C13" s="31" t="s">
-        <v>79</v>
+      <c r="C13" s="30" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14" s="35">
+        <v>74</v>
+      </c>
+      <c r="B14" s="34">
         <v>0.05</v>
       </c>
-      <c r="C14" s="31" t="s">
-        <v>81</v>
+      <c r="C14" s="30" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="36">
+        <v>76</v>
+      </c>
+      <c r="B15" s="35">
         <f>SUM(B12:B14)</f>
         <v>0.65000000000000013</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="37">
+        <v>77</v>
+      </c>
+      <c r="B17" s="36">
         <f>B8</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="36">
+        <v>78</v>
+      </c>
+      <c r="B18" s="35">
         <f>B15*B17</f>
         <v>0.65000000000000013</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="34">
+        <v>0.08</v>
+      </c>
+      <c r="C22" s="39" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="34">
+        <v>0.09</v>
+      </c>
+      <c r="C23" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B24" s="34">
+        <v>0.12</v>
+      </c>
+      <c r="C24" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="33" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="38" t="s">
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="35">
-        <v>0.08</v>
-      </c>
-      <c r="C22" s="40" t="s">
+      <c r="B25" s="34">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C25" s="39" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="38" t="s">
+    <row r="26" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="35">
-        <v>0.09</v>
-      </c>
-      <c r="C23" s="40" t="s">
+      <c r="B27" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="39" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="38" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="35">
-        <v>0.12</v>
-      </c>
-      <c r="C24" s="40" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="38" t="s">
-        <v>94</v>
-      </c>
-      <c r="B25" s="35">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="C25" s="40" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="38"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="38"/>
-    </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="C27" s="40" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="41" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="42">
+      <c r="B28" s="40">
         <f>INDEX(B22:B25,MATCH(B27,A22:A25,0))</f>
         <v>0.08</v>
       </c>
-      <c r="C28" s="38"/>
+      <c r="C28" s="37"/>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="38"/>
-      <c r="B29" s="43"/>
-      <c r="C29" s="38"/>
+      <c r="A29" s="37"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="37"/>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="41" t="s">
-        <v>99</v>
-      </c>
-      <c r="B30" s="42">
+      <c r="A30" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" s="40">
         <f>B18+B28</f>
         <v>0.73000000000000009</v>
       </c>
-      <c r="C30" s="38"/>
+      <c r="C30" s="37"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="B31" s="44">
+      <c r="A31" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" s="42">
         <f>B30/B7</f>
         <v>0.18250000000000002</v>
       </c>
-      <c r="C31" s="38"/>
+      <c r="C31" s="37"/>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1908,7 +2175,7 @@
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C33" t="s">
         <v>5</v>
@@ -1916,29 +2183,29 @@
     </row>
     <row r="34" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B34">
         <v>0.02</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B35">
         <v>0.01</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B36">
         <f>SUM(B34:B35)</f>
@@ -1946,292 +2213,292 @@
       </c>
     </row>
     <row r="37" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="41" t="s">
-        <v>107</v>
-      </c>
-      <c r="B37" s="42">
+      <c r="A37" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B37" s="40">
         <f>B36+B30</f>
         <v>0.76000000000000012</v>
       </c>
-      <c r="C37" s="38"/>
+      <c r="C37" s="37"/>
     </row>
     <row r="38" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="32" t="s">
+      <c r="A38" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
+    </row>
+    <row r="39" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="B39" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="B40" s="34">
+        <v>0.88</v>
+      </c>
+      <c r="C40" s="39" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="34">
+        <v>1.55</v>
+      </c>
+      <c r="C41" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="38"/>
-      <c r="C38" s="38"/>
-    </row>
-    <row r="39" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="33" t="s">
+    </row>
+    <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="B39" s="39" t="s">
+      <c r="B42" s="34">
+        <v>1.9</v>
+      </c>
+      <c r="C42" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="C39" s="33" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="38" t="s">
+    </row>
+    <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="B40" s="35">
-        <v>0.88</v>
-      </c>
-      <c r="C40" s="40" t="s">
+      <c r="B43" s="34">
+        <v>2.75</v>
+      </c>
+      <c r="C43" s="39" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="38" t="s">
+    <row r="44" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="B41" s="35">
-        <v>1.55</v>
-      </c>
-      <c r="C41" s="40" t="s">
+      <c r="B44" s="34">
+        <v>3.65</v>
+      </c>
+      <c r="C44" s="39" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="38" t="s">
+    <row r="45" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="B42" s="35">
-        <v>1.9</v>
-      </c>
-      <c r="C42" s="40" t="s">
+      <c r="B45" s="34">
+        <v>8.75</v>
+      </c>
+      <c r="C45" s="39" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="38" t="s">
+    <row r="46" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="37"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
+    </row>
+    <row r="47" spans="1:3" ht="81.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="B43" s="35">
-        <v>2.75</v>
-      </c>
-      <c r="C43" s="40" t="s">
+      <c r="B47" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="C47" s="39" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="38" t="s">
+    <row r="48" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B44" s="35">
-        <v>3.65</v>
-      </c>
-      <c r="C44" s="40" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="B45" s="35">
-        <v>8.75</v>
-      </c>
-      <c r="C45" s="40" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="38"/>
-      <c r="B46" s="38"/>
-      <c r="C46" s="38"/>
-    </row>
-    <row r="47" spans="1:3" ht="81.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="B47" s="35" t="s">
-        <v>113</v>
-      </c>
-      <c r="C47" s="40" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="B48" s="42">
+      <c r="B48" s="40">
         <f>INDEX(B40:B45,MATCH(B47,A40:A45,0))</f>
         <v>1.55</v>
       </c>
-      <c r="C48" s="38"/>
+      <c r="C48" s="37"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="38"/>
-      <c r="B49" s="43"/>
-      <c r="C49" s="38"/>
+      <c r="A49" s="37"/>
+      <c r="B49" s="41"/>
+      <c r="C49" s="37"/>
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="B50" s="38"/>
-      <c r="C50" s="38"/>
+      <c r="A50" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="B50" s="37"/>
+      <c r="C50" s="37"/>
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="33" t="s">
+      <c r="A51" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B51" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" s="33" t="s">
+      <c r="B51" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="C51" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="38" t="s">
-        <v>127</v>
-      </c>
-      <c r="B52" s="35">
+      <c r="A52" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="B52" s="34">
         <v>15.89</v>
       </c>
-      <c r="C52" s="40" t="s">
-        <v>128</v>
+      <c r="C52" s="39" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="38" t="s">
-        <v>129</v>
-      </c>
-      <c r="B53" s="35">
+      <c r="A53" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="B53" s="34">
         <v>25</v>
       </c>
-      <c r="C53" s="38"/>
+      <c r="C53" s="37"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="B54" s="42">
+      <c r="A54" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B54" s="40">
         <f>B52/B53</f>
         <v>0.63560000000000005</v>
       </c>
-      <c r="C54" s="38"/>
+      <c r="C54" s="37"/>
     </row>
     <row r="55" spans="1:3" ht="114.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="B55" s="35">
+      <c r="A55" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="B55" s="34">
         <v>3</v>
       </c>
-      <c r="C55" s="40" t="s">
-        <v>132</v>
+      <c r="C55" s="39" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
+      <c r="A56" s="51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B56" s="51"/>
+      <c r="C56" s="51"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="38"/>
-      <c r="B57" s="38"/>
-      <c r="C57" s="38"/>
+      <c r="A57" s="37"/>
+      <c r="B57" s="37"/>
+      <c r="C57" s="37"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="41" t="s">
-        <v>134</v>
-      </c>
-      <c r="B58" s="42">
+      <c r="A58" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B58" s="40">
         <f>B30+B48+B56+B36</f>
         <v>2.31</v>
       </c>
-      <c r="C58" s="38"/>
+      <c r="C58" s="37"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="38" t="s">
-        <v>135</v>
-      </c>
-      <c r="B59" s="44">
+      <c r="A59" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="B59" s="42">
         <f>B58/B7</f>
         <v>0.57750000000000001</v>
       </c>
-      <c r="C59" s="38"/>
+      <c r="C59" s="37"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="38"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="38"/>
+      <c r="A60" s="37"/>
+      <c r="B60" s="37"/>
+      <c r="C60" s="37"/>
     </row>
     <row r="61" spans="1:3" ht="186.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="40" t="s">
-        <v>136</v>
+      <c r="A61" s="39" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="32" t="s">
-        <v>137</v>
+      <c r="A63" s="31" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B64" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="C64" s="33" t="s">
+      <c r="B64" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C64" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="B65" s="45">
+      <c r="A65" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="B65" s="43">
         <f>'Recurring Overhead'!B32</f>
         <v>0</v>
       </c>
-      <c r="C65" s="46" t="s">
-        <v>139</v>
+      <c r="C65" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="B66" s="43">
+      <c r="A66" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B66" s="41">
         <f>B65*B7</f>
         <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="41" t="s">
-        <v>141</v>
-      </c>
-      <c r="B68" s="42">
+      <c r="A68" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B68" s="40">
         <f>B58+B66</f>
         <v>2.31</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="38" t="s">
-        <v>142</v>
-      </c>
-      <c r="B69" s="44">
+      <c r="A69" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="B69" s="42">
         <f>B68/B7</f>
         <v>0.57750000000000001</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
+      <c r="A71" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="B71" s="52"/>
+      <c r="C71" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2256,264 +2523,264 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" s="18">
+        <v>0</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="B7" s="18">
+        <v>0</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="17" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="B8" s="18">
+        <v>0</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="19">
+      <c r="D8" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="B9" s="18">
         <v>0</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="18" t="s">
+      <c r="C9" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B7" s="19">
-        <v>0</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="D7" s="5" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="19" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="B8" s="19">
-        <v>0</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="19">
-        <v>0</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="21">
+      <c r="B10" s="20">
         <f>SUM(B6:B9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="50" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="50"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="17" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B16" s="44">
+        <v>10</v>
+      </c>
+      <c r="C16" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="17" t="s">
+      <c r="D16" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B15" s="17" t="s">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="B17" s="44">
+        <v>40</v>
+      </c>
+      <c r="C17" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D17" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="18" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="B16" s="47">
-        <v>10</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="B17" s="47">
-        <v>40</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="B18" s="48">
+      <c r="B18" s="45">
         <f>B20</f>
         <v>0</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>173</v>
+      <c r="C18" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="B20" s="49">
+      <c r="A20" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="46">
         <v>0</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>175</v>
+      <c r="D20" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="B21" s="48">
+      <c r="A21" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="B21" s="45">
         <f>IFERROR(B20*4.33/(45/60)*20,0)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>177</v>
+      <c r="D21" s="1" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
-        <v>178</v>
+      <c r="A23" s="12" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>179</v>
+      <c r="A24" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="B25" s="28">
+      <c r="A25" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" s="27">
         <f>IFERROR($B$10/B16,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="B26" s="28">
+      <c r="A26" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="B26" s="27">
         <f>IFERROR($B$10/B17,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="B27" s="28">
+      <c r="A27" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B27" s="27">
         <f>IFERROR($B$10/B18,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
-        <v>180</v>
+      <c r="A29" s="12" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="B30" s="50" t="s">
-        <v>165</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>182</v>
+      <c r="A30" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="B31" s="48">
+      <c r="A31" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B31" s="45">
         <f>INDEX(B16:B18,MATCH(B30,A16:A18,0))</f>
         <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="20" t="s">
-        <v>184</v>
-      </c>
-      <c r="B32" s="21">
+      <c r="A32" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B32" s="20">
         <f>IFERROR($B$10/B31,0)</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add new business plan document for custom sticker side hustle and update StickerBinStickersCosts v2.xlsx
- Introduced a comprehensive business plan for producing custom vinyl stickers, detailing market overview, product offerings, legal considerations, and startup costs.
- Updated the StickerBinStickersCosts v2.xlsx file to reflect revised cost data.

This commit enhances the project documentation and provides a strategic framework for the sticker business initiative.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED96A0C-EAFE-4268-9582-A79529B7C103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD330459-99FD-4F8C-892E-18FE9514D80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -466,16 +466,10 @@
     <t>Cost (£/month)</t>
   </si>
   <si>
-    <t>Design software (e.g. Canva Pro, Adobe, Procreate — TBD)</t>
-  </si>
-  <si>
     <t>Design</t>
   </si>
   <si>
     <t>Placeholder — not yet chosen (per chat, July 2026). Separate from Midjourney, already costed per-design-set in the Business Plan; add it here too if it becomes an ongoing monthly subscription.</t>
-  </si>
-  <si>
-    <t>Font licences</t>
   </si>
   <si>
     <t>Placeholder — for any paid/commercial-use fonts beyond free/open-license options.</t>
@@ -648,6 +642,12 @@
   <si>
     <t>cricut</t>
   </si>
+  <si>
+    <t>Midjourney </t>
+  </si>
+  <si>
+    <t>lovart</t>
+  </si>
 </sst>
 </file>
 
@@ -657,7 +657,7 @@
     <numFmt numFmtId="164" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -836,6 +836,18 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -891,7 +903,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -948,11 +960,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1278,7 +1292,7 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1295,7 +1309,7 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1312,7 +1326,7 @@
         <v>14</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1373,7 +1387,7 @@
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="49" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B13">
         <v>4</v>
@@ -1518,12 +1532,12 @@
         <v>5</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" x14ac:dyDescent="0.35">
-      <c r="A31" s="53" t="s">
-        <v>183</v>
+      <c r="A31" s="50" t="s">
+        <v>181</v>
       </c>
       <c r="B31" s="18">
         <v>13</v>
@@ -1538,12 +1552,12 @@
         <v>0.52</v>
       </c>
       <c r="G31" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" x14ac:dyDescent="0.35">
-      <c r="A32" s="53" t="s">
-        <v>184</v>
+      <c r="A32" s="50" t="s">
+        <v>182</v>
       </c>
       <c r="B32" s="18">
         <v>8</v>
@@ -1558,16 +1572,16 @@
         <v>10</v>
       </c>
       <c r="F32">
-        <f t="shared" ref="F32:F42" si="0">B32/E32</f>
+        <f t="shared" ref="F32:F40" si="0">B32/E32</f>
         <v>0.8</v>
       </c>
       <c r="G32" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" x14ac:dyDescent="0.35">
-      <c r="A33" s="53" t="s">
-        <v>185</v>
+      <c r="A33" s="50" t="s">
+        <v>183</v>
       </c>
       <c r="B33" s="18">
         <v>5.85</v>
@@ -1586,12 +1600,12 @@
         <v>0.58499999999999996</v>
       </c>
       <c r="G33" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="54" t="s">
-        <v>186</v>
+      <c r="A34" s="51" t="s">
+        <v>184</v>
       </c>
       <c r="B34" s="18">
         <v>6</v>
@@ -1606,12 +1620,12 @@
         <v>0.24</v>
       </c>
       <c r="G34" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="54" t="s">
-        <v>187</v>
+      <c r="A35" s="51" t="s">
+        <v>185</v>
       </c>
       <c r="B35" s="18">
         <v>7.37</v>
@@ -1626,12 +1640,12 @@
         <v>0.1474</v>
       </c>
       <c r="G35" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="54" t="s">
-        <v>188</v>
+      <c r="A36" s="51" t="s">
+        <v>186</v>
       </c>
       <c r="B36" s="18">
         <v>6</v>
@@ -1646,12 +1660,12 @@
         <v>0.24</v>
       </c>
       <c r="G36" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="54" t="s">
-        <v>189</v>
+      <c r="A37" s="51" t="s">
+        <v>187</v>
       </c>
       <c r="B37" s="18">
         <v>9</v>
@@ -1666,12 +1680,12 @@
         <v>0.09</v>
       </c>
       <c r="G37" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="54" t="s">
-        <v>190</v>
+      <c r="A38" s="51" t="s">
+        <v>188</v>
       </c>
       <c r="B38" s="18">
         <v>5</v>
@@ -1686,12 +1700,12 @@
         <v>0.125</v>
       </c>
       <c r="G38" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="54" t="s">
-        <v>191</v>
+      <c r="A39" s="51" t="s">
+        <v>189</v>
       </c>
       <c r="B39" s="18">
         <v>6.09</v>
@@ -1706,12 +1720,12 @@
         <v>0.60899999999999999</v>
       </c>
       <c r="G39" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="54" t="s">
-        <v>192</v>
+      <c r="A40" s="51" t="s">
+        <v>190</v>
       </c>
       <c r="B40" s="18">
         <v>10</v>
@@ -1726,12 +1740,12 @@
         <v>0.2</v>
       </c>
       <c r="G40" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B41" s="18">
         <v>13</v>
@@ -1746,10 +1760,10 @@
         <v>0.85</v>
       </c>
       <c r="G41" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H41" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I41">
         <v>4</v>
@@ -1757,7 +1771,7 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B42" s="18">
         <v>13</v>
@@ -1772,10 +1786,10 @@
         <v>0.85</v>
       </c>
       <c r="G42" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H42" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="I42">
         <v>4</v>
@@ -1800,12 +1814,12 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="50" t="s">
+      <c r="A46" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="50"/>
-      <c r="C46" s="50"/>
-      <c r="D46" s="50"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="52"/>
+      <c r="D46" s="52"/>
     </row>
     <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="23" t="s">
@@ -1813,12 +1827,12 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="50" t="s">
+      <c r="A49" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="50"/>
-      <c r="C49" s="50"/>
-      <c r="D49" s="50"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="52"/>
+      <c r="D49" s="52"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
@@ -1837,7 +1851,7 @@
       </c>
       <c r="B52" s="24">
         <f>'Bin Stickers 100x150 4pk'!B68</f>
-        <v>2.31</v>
+        <v>23.506</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>51</v>
@@ -1849,7 +1863,7 @@
       </c>
       <c r="B53" s="26">
         <f>B51-B52</f>
-        <v>3.69</v>
+        <v>-17.506</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -1867,7 +1881,7 @@
       </c>
       <c r="B56" s="28">
         <f>IFERROR(B55/B53,"N/A")</f>
-        <v>171.08672086720867</v>
+        <v>-36.062492859590996</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -1876,16 +1890,16 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56*'Bin Stickers 100x150 4pk'!B7,"N/A")</f>
-        <v>684.34688346883468</v>
+        <v>-144.24997143836399</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="50" t="s">
+      <c r="A59" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="B59" s="50"/>
-      <c r="C59" s="50"/>
-      <c r="D59" s="50"/>
+      <c r="B59" s="52"/>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2397,11 +2411,11 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="51" t="s">
+      <c r="A56" s="53" t="s">
         <v>127</v>
       </c>
-      <c r="B56" s="51"/>
-      <c r="C56" s="51"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="53"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="37"/>
@@ -2460,7 +2474,7 @@
       </c>
       <c r="B65" s="43">
         <f>'Recurring Overhead'!B32</f>
-        <v>0</v>
+        <v>5.2990000000000004</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>133</v>
@@ -2472,7 +2486,7 @@
       </c>
       <c r="B66" s="41">
         <f>B65*B7</f>
-        <v>0</v>
+        <v>21.196000000000002</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -2481,7 +2495,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>2.31</v>
+        <v>23.506</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2490,15 +2504,15 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>0.57750000000000001</v>
+        <v>5.8765000000000001</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="52" t="s">
+      <c r="A71" s="54" t="s">
         <v>137</v>
       </c>
-      <c r="B71" s="52"/>
-      <c r="C71" s="52"/>
+      <c r="B71" s="54"/>
+      <c r="C71" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2527,12 +2541,12 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
@@ -2553,223 +2567,223 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="55" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="18">
+        <v>8.9</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="B6" s="18">
-        <v>0</v>
-      </c>
-      <c r="C6" s="17" t="s">
+      <c r="D6" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="56" t="s">
+        <v>198</v>
+      </c>
+      <c r="B7" s="18">
+        <v>14.09</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>144</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="B7" s="18">
-        <v>0</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="B8" s="18">
+        <v>30</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="B8" s="18">
-        <v>0</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B9" s="18">
         <v>0</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B10" s="20">
         <f>SUM(B6:B9)</f>
-        <v>0</v>
+        <v>52.99</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="50" t="s">
-        <v>154</v>
-      </c>
-      <c r="B13" s="50"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
+      <c r="A13" s="52" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="D15" s="16" t="s">
         <v>156</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B16" s="44">
         <v>10</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B17" s="44">
         <v>40</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B18" s="45">
         <f>B20</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B20" s="46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B21" s="45">
         <f>IFERROR(B20*4.33/(45/60)*20,0)</f>
-        <v>0</v>
+        <v>115.46666666666667</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B25" s="27">
         <f>IFERROR($B$10/B16,0)</f>
-        <v>0</v>
+        <v>5.2990000000000004</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B26" s="27">
         <f>IFERROR($B$10/B17,0)</f>
-        <v>0</v>
+        <v>1.3247500000000001</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B27" s="27">
         <f>IFERROR($B$10/B18,0)</f>
-        <v>0</v>
+        <v>52.99</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="17" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B30" s="47" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="17" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B31" s="45">
         <f>INDEX(B16:B18,MATCH(B30,A16:A18,0))</f>
@@ -2778,11 +2792,11 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="19" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B32" s="20">
         <f>IFERROR($B$10/B31,0)</f>
-        <v>0</v>
+        <v>5.2990000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add marketing guides for Amazon, eBay, and Etsy
- Created new reference guides for Amazon, eBay, and Etsy marketing strategies tailored for the Bin Sticker Side Hustle.
- Each guide includes detailed fee structures, advertising options, and recommended launch approaches, ensuring comprehensive preparation for future sales channels.
- Emphasized the importance of verifying current rates and conditions before implementation, reflecting the dynamic nature of each platform's policies.

These additions provide essential insights for effective marketing and cost management across multiple e-commerce platforms.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DEA2AA-DBD7-4CF8-B175-E31FC812AB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3005BDE-59F1-4C40-B908-0B40CD916460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
     <sheet name="Bin Stickers 100x140 4pk" sheetId="2" r:id="rId2"/>
     <sheet name="Recurring Overhead" sheetId="3" r:id="rId3"/>
+    <sheet name="cost per item" sheetId="4" r:id="rId4"/>
+    <sheet name="Ebay costs" sheetId="5" r:id="rId5"/>
+    <sheet name="Etsy" sheetId="6" r:id="rId6"/>
+    <sheet name="Amazon" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="304">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -638,17 +642,327 @@
   </si>
   <si>
     <t>full year</t>
+  </si>
+  <si>
+    <t>item</t>
+  </si>
+  <si>
+    <t>cost</t>
+  </si>
+  <si>
+    <t>shipping</t>
+  </si>
+  <si>
+    <t>total per item</t>
+  </si>
+  <si>
+    <t>Stickiply</t>
+  </si>
+  <si>
+    <t>white vinyl</t>
+  </si>
+  <si>
+    <t>clear vinyl</t>
+  </si>
+  <si>
+    <t>lamination</t>
+  </si>
+  <si>
+    <t>Cricut</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>per item</t>
+  </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>EBAY MARKETING — PROMOTED LISTINGS &amp; FEE STACK (added Aug 2026)</t>
+  </si>
+  <si>
+    <t>Ad spend is a VARIABLE cost (scales with price × volume), unlike the fixed monthly subscriptions above — deliberately kept as its own block rather than folded into the MONTHLY OVERHEAD SUBTOTAL (B11), since mixing a %-of-price cost into that flat per-sticker allocation would distort it whenever price changes. See chat for full research: ad-rate benchmarks, eBay's own suggested rates vs independent guidance, and how this stacks with Final Value Fee / per-order fee / regulatory fee. FLAG: price input below (£3.00) is a placeholder mid-point of the user-specified £2-4 'simple stickers' range (Aug 2026 chat) — this differs from the Business Plan Section 3 bin sticker range (£5-8/set) and the 'Bin Stickers 100x140 4pk' sheet (~£6/pack). Clarify whether this is a new single-sticker product tier or a per-unit breakdown of the existing set price, then reconcile across files.</t>
+  </si>
+  <si>
+    <t>Assumed sale price per unit (£)</t>
+  </si>
+  <si>
+    <t>Placeholder mid-point of user-specified £2-4 range — see flag above. Edit once price is locked.</t>
+  </si>
+  <si>
+    <t>Promoted Listings ad rate (% of sale price)</t>
+  </si>
+  <si>
+    <t>User-selected 4% (Aug 2026 chat) — independent-guidance recommended ceiling for small/new sellers. eBay's own suggested rate typically runs 8-15% and is optimised for eBay's revenue, not yours; community reports of 2-30% exist depending on category/margin. General/Standard campaign (cost-per-sale) assumed, not Priority/Advanced (cost-per-click) — right choice for a single-product launch at this volume.</t>
+  </si>
+  <si>
+    <t>eBay Final Value Fee (business seller, standard category)</t>
+  </si>
+  <si>
+    <t>12.8% of item price + postage, most categories, checked Aug 2026. Matches the ~13% already assumed in Business Plan Section 6, just broken out precisely here.</t>
+  </si>
+  <si>
+    <t>eBay per-order fee (£, flat)</t>
+  </si>
+  <si>
+    <t>30p per order under £10; rises to 40p for orders ≥£10 (changed Feb 2026 — NOT yet reflected in Business Plan Section 6 or the 4pk cost sheet, worth adding there too). At a £2-4 unit price this stays at 30p unless bundling pushes a single order over £10.</t>
+  </si>
+  <si>
+    <t>eBay Regulatory Operating Fee (% of item price + postage)</t>
+  </si>
+  <si>
+    <t>~0.35-0.43% UK regulatory fee, introduced April 2024, applies to all UK business sellers regardless of ad usage — also not currently broken out elsewhere in the workbook. 0.4% used as a midpoint.</t>
+  </si>
+  <si>
+    <t>→ COST PER UNIT SOLD</t>
+  </si>
+  <si>
+    <t>Ad spend per unit (£)</t>
+  </si>
+  <si>
+    <t>Final Value Fee per unit (£)</t>
+  </si>
+  <si>
+    <t>Regulatory fee per unit (£)</t>
+  </si>
+  <si>
+    <t>TOTAL EBAY PLATFORM COST PER UNIT (FVF + per-order + regulatory + ad) (£)</t>
+  </si>
+  <si>
+    <t>Net proceeds per unit after all eBay fees (£)</t>
+  </si>
+  <si>
+    <t>Total eBay fees as % of sale price</t>
+  </si>
+  <si>
+    <t>→ MONTHLY, AT ACTIVE SCENARIO VOLUME (from ACTIVE SCENARIO block above)</t>
+  </si>
+  <si>
+    <t>Active monthly volume (stickers)</t>
+  </si>
+  <si>
+    <t>Monthly ad spend at active volume (£)</t>
+  </si>
+  <si>
+    <t>Monthly TOTAL eBay platform fees at active volume (£)</t>
+  </si>
+  <si>
+    <t>Not yet wired into the per-sticker OVERHEAD figures above (B26-B33) or into the 'Bin Stickers 100x140 4pk' sheet, on purpose — it's a %-of-price cost, and that sheet models a different price point (£6/4pk) than the £2-4 range given here. Once the 'simple stickers' price/product is confirmed, this block's TOTAL EBAY PLATFORM COST PER UNIT row can be added directly into that sheet's fee/margin table, or this section's monthly ad spend can be added into B11's SUM range above if you'd rather treat it as pooled overhead — flag either way so the two stay consistent.</t>
+  </si>
+  <si>
+    <t>Etsy — Fees &amp; Advertising (UK shop, not VAT-registered)</t>
+  </si>
+  <si>
+    <t>Blue = editable input. Black = calculated. Companion to Etsy-Marketing-Guide.md — see that file for full context/sources. FLAG: price input below (£3.00) is a placeholder mid-point of the user-specified £2-4 'simple stickers' range — differs from Business Plan Section 3 (£5-8/set bin stickers). 'Sale price' here is treated as the TOTAL amount the buyer pays (item + any shipping charged), matching how Etsy calculates its fees.</t>
+  </si>
+  <si>
+    <t>INPUTS</t>
+  </si>
+  <si>
+    <t>Assumed sale price per unit, total incl. shipping (£)</t>
+  </si>
+  <si>
+    <t>Placeholder — see flag above. Edit once price is locked.</t>
+  </si>
+  <si>
+    <t>Listing fee per listing (£)</t>
+  </si>
+  <si>
+    <t>~$0.20 USD converted. Charged whether or not it sells; renews every 4 months and again per sale on multi-quantity listings — this model assumes 1 listing fee per unit sold, the conservative case.</t>
+  </si>
+  <si>
+    <t>Transaction fee rate</t>
+  </si>
+  <si>
+    <t>6.5% of item price + shipping + gift wrap.</t>
+  </si>
+  <si>
+    <t>Payment processing rate</t>
+  </si>
+  <si>
+    <t>4% + fixed fee below. Etsy Payments is mandatory, no alternative processor option.</t>
+  </si>
+  <si>
+    <t>Payment processing fixed fee (£)</t>
+  </si>
+  <si>
+    <t>Regulatory Operating Fee rate</t>
+  </si>
+  <si>
+    <t>0.32% of item price + shipping, UK-specific since 2022.</t>
+  </si>
+  <si>
+    <t>VAT on Etsy fees (applies — not VAT-registered)</t>
+  </si>
+  <si>
+    <t>20% VAT charged on ALL of Etsy's fees above when the seller isn't VAT-registered (per current business plan strategy). Set to 0% here if VAT registration status changes.</t>
+  </si>
+  <si>
+    <t>Offsite Ads currently active? (Y/N)</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Optional and should be switched OFF in Shop Manager while trailing 12-month revenue is under $10,000 USD (~£8,000) — see guide. Becomes mandatory (can't be set to N) once that threshold is crossed.</t>
+  </si>
+  <si>
+    <t>Offsite Ads fee rate (if active)</t>
+  </si>
+  <si>
+    <t>15% below $10k trailing revenue, 12% once mandatory at/above it.</t>
+  </si>
+  <si>
+    <t>Etsy Ads (onsite) daily budget (£) — optional, separate CPC spend</t>
+  </si>
+  <si>
+    <t>Minimum ~£1/day. This is a controllable CPC budget, NOT a %-of-sale fee — kept separate from the cost-per-unit maths below since it doesn't scale with units sold. Shown as a monthly figure further down.</t>
+  </si>
+  <si>
+    <t>→ COST PER UNIT SOLD (Listing + Transaction + Payment processing + Regulatory + VAT-on-fees)</t>
+  </si>
+  <si>
+    <t>Transaction fee (£)</t>
+  </si>
+  <si>
+    <t>Payment processing fee (£)</t>
+  </si>
+  <si>
+    <t>Regulatory fee (£)</t>
+  </si>
+  <si>
+    <t>Subtotal before VAT (£)</t>
+  </si>
+  <si>
+    <t>VAT on fees (£)</t>
+  </si>
+  <si>
+    <t>Offsite Ads fee incl. its own VAT (£), if active</t>
+  </si>
+  <si>
+    <t>TOTAL ETSY FEES PER UNIT (£)</t>
+  </si>
+  <si>
+    <t>Net proceeds per unit after all Etsy fees (£)</t>
+  </si>
+  <si>
+    <t>Total Etsy fees as % of sale price</t>
+  </si>
+  <si>
+    <t>→ MONTHLY, AT ACTIVE SCENARIO VOLUME (from 'Recurring Overhead' sheet)</t>
+  </si>
+  <si>
+    <t>Monthly total Etsy fees at active volume (£)</t>
+  </si>
+  <si>
+    <t>Monthly Etsy Ads (onsite) budget, if used (£)</t>
+  </si>
+  <si>
+    <t>Independent of units sold — a controllable CPC budget, not charged per unit.</t>
+  </si>
+  <si>
+    <t>Not wired into the 'Recurring Overhead' sheet's fixed subscription subtotal (B11), same rationale as the eBay block there: these are %-of-price/variable costs, and mixing them into a flat £/sticker overhead figure would distort it whenever price changes. See Etsy-Marketing-Guide.md for the recommended launch approach (Offsite Ads off, small onsite Ads budget, fix listing fundamentals first).</t>
+  </si>
+  <si>
+    <t>Amazon — Fees &amp; Advertising (UK, FBM assumed)</t>
+  </si>
+  <si>
+    <t>Blue = editable input. Black = calculated. Companion to Amazon-Marketing-Guide.md. FLAG: same £2-4 vs £5-8 price ambiguity as the other sheets applies here — £3.00 used as a placeholder. Amazon Handmade eligibility (12.24% flat referral fee, vs standard 8-15% category fee) is NOT confirmed for laminated vinyl stickers — standard referral fee used below as the conservative default; switch the input if Handmade is confirmed eligible.</t>
+  </si>
+  <si>
+    <t>Placeholder — see flag above.</t>
+  </si>
+  <si>
+    <t>Referral fee rate</t>
+  </si>
+  <si>
+    <t>8-15% typical range by category; 15% (top of range) used as the conservative default. Confirm actual category rate before launch — check Amazon Handmade (12.24% flat) eligibility too.</t>
+  </si>
+  <si>
+    <t>Minimum referral fee (£)</t>
+  </si>
+  <si>
+    <t>Applies regardless of price — matters at £2-4 unit prices since the percentage-based fee may fall below this floor.</t>
+  </si>
+  <si>
+    <t>Digital Services Tax pass-through rate</t>
+  </si>
+  <si>
+    <t>Applied on top of the referral fee for UK-established sellers.</t>
+  </si>
+  <si>
+    <t>Using Professional account? (Y/N)</t>
+  </si>
+  <si>
+    <t>Required for Sponsored Products (PPC) access, Buy Box eligibility, and new listing creation. Guide recommends holding off until volume/margin justify the flat monthly cost. Set to 'Y' once committed.</t>
+  </si>
+  <si>
+    <t>Professional account monthly fee (£)</t>
+  </si>
+  <si>
+    <t>Individual account per-item fee (£, if not Professional)</t>
+  </si>
+  <si>
+    <t>Sponsored Products target ACoS (launch phase)</t>
+  </si>
+  <si>
+    <t>30-40%+ is normal/accepted during a launch phase per general guidance; established-product benchmarks run 15-25%. Only relevant if Professional account + Sponsored Products are actually turned on.</t>
+  </si>
+  <si>
+    <t>→ COST PER UNIT SOLD (selling fees only, before advertising)</t>
+  </si>
+  <si>
+    <t>Referral fee, greater of rate or minimum (£)</t>
+  </si>
+  <si>
+    <t>Referral fee incl. DST pass-through (£)</t>
+  </si>
+  <si>
+    <t>Account fee per unit — Individual only (£)</t>
+  </si>
+  <si>
+    <t>Professional's £25/mo is a flat monthly cost, not per-unit — shown separately below.</t>
+  </si>
+  <si>
+    <t>TOTAL SELLING FEES PER UNIT (£)</t>
+  </si>
+  <si>
+    <t>Net proceeds per unit after selling fees, before advertising (£)</t>
+  </si>
+  <si>
+    <t>Total selling fees as % of sale price</t>
+  </si>
+  <si>
+    <t>→ MONTHLY, AT ACTIVE SCENARIO VOLUME</t>
+  </si>
+  <si>
+    <t>Monthly total selling fees at active volume (£)</t>
+  </si>
+  <si>
+    <t>Monthly Professional account fee, if used (£)</t>
+  </si>
+  <si>
+    <t>Estimated monthly Sponsored Products spend, if Professional + advertising used (£)</t>
+  </si>
+  <si>
+    <t>Approximation: ACoS × assumed monthly revenue, treating all volume as ad-attributed — a simplification, real ad-attributed revenue will be a subset of total sales. CPC spend is NOT cost-per-sale, so this is charged whether or not those specific clicks convert.</t>
+  </si>
+  <si>
+    <t>Not wired into the 'Recurring Overhead' sheet's fixed subscription subtotal (B11) — same rationale as the eBay and Etsy blocks: variable/%-of-price costs kept separate from the flat £/sticker overhead allocation. Guide recommends holding Professional account + Sponsored Products off until Amazon volume and margin are established via eBay/Etsy first — the Y/N toggles above default to 'off' accordingly.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -832,8 +1146,48 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF666666"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF1F3864"/>
+      <name val="Cambria"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -856,6 +1210,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1F1F1F"/>
       </patternFill>
     </fill>
   </fills>
@@ -887,7 +1253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -948,10 +1314,43 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1799,12 +2198,12 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="57" t="s">
+      <c r="A46" s="64" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="55"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
+      <c r="B46" s="65"/>
+      <c r="C46" s="65"/>
+      <c r="D46" s="65"/>
     </row>
     <row r="48" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="23" t="s">
@@ -1812,12 +2211,12 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="57" t="s">
+      <c r="A49" s="64" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="55"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
+      <c r="B49" s="65"/>
+      <c r="C49" s="65"/>
+      <c r="D49" s="65"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
@@ -1836,7 +2235,7 @@
       </c>
       <c r="B52" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
-        <v>27.826000000000001</v>
+        <v>28.337866666666667</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>112</v>
@@ -1848,7 +2247,7 @@
       </c>
       <c r="B53" s="26">
         <f>B51-B52</f>
-        <v>-21.826000000000001</v>
+        <v>-22.337866666666667</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -1866,7 +2265,7 @@
       </c>
       <c r="B56" s="28">
         <f>IFERROR(B55/B53,"N/A")</f>
-        <v>-28.924676990744981</v>
+        <v>-28.261875201451645</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -1875,16 +2274,16 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
-        <v>-115.69870796297992</v>
+        <v>-113.04750080580658</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="57" t="s">
+      <c r="A59" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="B59" s="55"/>
-      <c r="C59" s="55"/>
-      <c r="D59" s="55"/>
+      <c r="B59" s="65"/>
+      <c r="C59" s="65"/>
+      <c r="D59" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2007,7 +2406,7 @@
         <v>133</v>
       </c>
       <c r="B13" s="34">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="C13" s="30" t="s">
         <v>134</v>
@@ -2030,7 +2429,7 @@
       </c>
       <c r="B15" s="35">
         <f>SUM(B12:B14)</f>
-        <v>0.65000000000000013</v>
+        <v>0.95000000000000007</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2048,7 +2447,7 @@
       </c>
       <c r="B18" s="35">
         <f>B15*B17</f>
-        <v>0.65000000000000013</v>
+        <v>0.95000000000000007</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2150,7 +2549,7 @@
       </c>
       <c r="B30" s="40">
         <f>B18+B28</f>
-        <v>0.73000000000000009</v>
+        <v>1.03</v>
       </c>
       <c r="C30" s="37"/>
     </row>
@@ -2160,7 +2559,7 @@
       </c>
       <c r="B31" s="42">
         <f>B30/B7</f>
-        <v>0.18250000000000002</v>
+        <v>0.25750000000000001</v>
       </c>
       <c r="C31" s="37"/>
     </row>
@@ -2217,7 +2616,7 @@
       </c>
       <c r="B37" s="40">
         <f>B36+B30</f>
-        <v>0.76000000000000012</v>
+        <v>1.06</v>
       </c>
       <c r="C37" s="37"/>
     </row>
@@ -2396,11 +2795,13 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="54" t="s">
+      <c r="A56" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B56" s="55"/>
-      <c r="C56" s="55"/>
+      <c r="B56">
+        <f>B54/3</f>
+        <v>0.21186666666666668</v>
+      </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="37"/>
@@ -2413,7 +2814,7 @@
       </c>
       <c r="B58" s="40">
         <f>B30+B48+B56+B36</f>
-        <v>1.6700000000000002</v>
+        <v>2.1818666666666666</v>
       </c>
       <c r="C58" s="37"/>
     </row>
@@ -2423,7 +2824,7 @@
       </c>
       <c r="B59" s="42">
         <f>B58/B7</f>
-        <v>0.41750000000000004</v>
+        <v>0.54546666666666666</v>
       </c>
       <c r="C59" s="37"/>
     </row>
@@ -2480,7 +2881,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>27.826000000000001</v>
+        <v>28.337866666666667</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2489,19 +2890,18 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>6.9565000000000001</v>
+        <v>7.0844666666666667</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="56" t="s">
+      <c r="A71" s="66" t="s">
         <v>198</v>
       </c>
-      <c r="B71" s="55"/>
-      <c r="C71" s="55"/>
+      <c r="B71" s="65"/>
+      <c r="C71" s="65"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A56:C56"/>
+  <mergeCells count="1">
     <mergeCell ref="A71:C71"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2526,12 +2926,12 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
@@ -2656,12 +3056,12 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="57" t="s">
+      <c r="A14" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
+      <c r="B14" s="65"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
@@ -2831,4 +3231,1239 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2EB3B2-BEC6-4259-8327-12EE41C40AEF}">
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E1" t="s">
+        <v>204</v>
+      </c>
+      <c r="I1" t="s">
+        <v>210</v>
+      </c>
+      <c r="J1" t="s">
+        <v>84</v>
+      </c>
+      <c r="K1" t="s">
+        <v>210</v>
+      </c>
+      <c r="L1" t="s">
+        <v>211</v>
+      </c>
+      <c r="M1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>6.5</v>
+      </c>
+      <c r="E3">
+        <f>C3/B3</f>
+        <v>0.65</v>
+      </c>
+      <c r="I3" t="s">
+        <v>206</v>
+      </c>
+      <c r="J3">
+        <v>25</v>
+      </c>
+      <c r="K3">
+        <f>C4+C14</f>
+        <v>25.9</v>
+      </c>
+      <c r="L3">
+        <f>K3/J3</f>
+        <v>1.036</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B4">
+        <v>25</v>
+      </c>
+      <c r="C4">
+        <v>13.25</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E22" si="0">C4/B4</f>
+        <v>0.53</v>
+      </c>
+      <c r="I4" t="s">
+        <v>206</v>
+      </c>
+      <c r="J4">
+        <v>50</v>
+      </c>
+      <c r="K4">
+        <f>C5+C15</f>
+        <v>46.15</v>
+      </c>
+      <c r="L4">
+        <f t="shared" ref="L4:L12" si="1">K4/J4</f>
+        <v>0.92299999999999993</v>
+      </c>
+      <c r="M4">
+        <f>L3-L4</f>
+        <v>0.1130000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5">
+        <v>50</v>
+      </c>
+      <c r="C5">
+        <v>22.5</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>0.45</v>
+      </c>
+      <c r="I5" t="s">
+        <v>206</v>
+      </c>
+      <c r="J5">
+        <v>100</v>
+      </c>
+      <c r="K5">
+        <f>C6+C16</f>
+        <v>87</v>
+      </c>
+      <c r="L5" s="54">
+        <f t="shared" si="1"/>
+        <v>0.87</v>
+      </c>
+      <c r="M5">
+        <f t="shared" ref="M5:M12" si="2">L4-L5</f>
+        <v>5.2999999999999936E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6">
+        <v>100</v>
+      </c>
+      <c r="C6">
+        <v>43</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>0.43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>206</v>
+      </c>
+      <c r="J6">
+        <v>200</v>
+      </c>
+      <c r="K6">
+        <f>C7+C17</f>
+        <v>165.5</v>
+      </c>
+      <c r="L6">
+        <f>K6/J6</f>
+        <v>0.82750000000000001</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="2"/>
+        <v>4.2499999999999982E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7">
+        <v>200</v>
+      </c>
+      <c r="C7">
+        <v>80</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>0.4</v>
+      </c>
+      <c r="I7" t="s">
+        <v>206</v>
+      </c>
+      <c r="J7">
+        <v>500</v>
+      </c>
+      <c r="K7">
+        <f>C8+C18</f>
+        <v>384</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="1"/>
+        <v>0.76800000000000002</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="2"/>
+        <v>5.9499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B8">
+        <v>500</v>
+      </c>
+      <c r="C8">
+        <v>175</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>0.35</v>
+      </c>
+      <c r="I8" t="s">
+        <v>207</v>
+      </c>
+      <c r="J8">
+        <v>25</v>
+      </c>
+      <c r="K8">
+        <f>C10+C14</f>
+        <v>28.9</v>
+      </c>
+      <c r="L8">
+        <f>K8/J8</f>
+        <v>1.1559999999999999</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="2"/>
+        <v>-0.3879999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>7.5</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>0.75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9">
+        <v>50</v>
+      </c>
+      <c r="K9">
+        <f>C11+C15</f>
+        <v>51.15</v>
+      </c>
+      <c r="L9">
+        <f>K9/J9</f>
+        <v>1.0229999999999999</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="2"/>
+        <v>0.13300000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>16.25</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>0.65</v>
+      </c>
+      <c r="I10" t="s">
+        <v>207</v>
+      </c>
+      <c r="J10">
+        <v>100</v>
+      </c>
+      <c r="K10">
+        <f>C12+C16</f>
+        <v>92</v>
+      </c>
+      <c r="L10" s="54">
+        <f>K10/J10</f>
+        <v>0.92</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="2"/>
+        <v>0.10299999999999987</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>50</v>
+      </c>
+      <c r="C11">
+        <v>27.5</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="I11" t="s">
+        <v>207</v>
+      </c>
+      <c r="J11">
+        <v>200</v>
+      </c>
+      <c r="K11">
+        <f>2*C12+C17</f>
+        <v>181.5</v>
+      </c>
+      <c r="L11">
+        <f>K11/J11</f>
+        <v>0.90749999999999997</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="2"/>
+        <v>1.2500000000000067E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>100</v>
+      </c>
+      <c r="C12">
+        <v>48</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>0.48</v>
+      </c>
+      <c r="I12" t="s">
+        <v>207</v>
+      </c>
+      <c r="J12">
+        <v>500</v>
+      </c>
+      <c r="K12">
+        <f>5*C12+C18</f>
+        <v>449</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="1"/>
+        <v>0.89800000000000002</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="2"/>
+        <v>9.4999999999999529E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>208</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13">
+        <v>5.5</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="I13" t="s">
+        <v>209</v>
+      </c>
+      <c r="J13">
+        <v>20</v>
+      </c>
+      <c r="K13">
+        <f>C20+C22</f>
+        <v>13</v>
+      </c>
+      <c r="L13">
+        <f>K13/J13</f>
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>12.65</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>0.50600000000000001</v>
+      </c>
+      <c r="I14" t="s">
+        <v>209</v>
+      </c>
+      <c r="J14">
+        <v>60</v>
+      </c>
+      <c r="K14">
+        <f>K13*3</f>
+        <v>39</v>
+      </c>
+      <c r="L14">
+        <f>K14/J14</f>
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>50</v>
+      </c>
+      <c r="C15">
+        <v>23.65</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>0.47299999999999998</v>
+      </c>
+      <c r="I15" t="s">
+        <v>209</v>
+      </c>
+      <c r="J15">
+        <v>100</v>
+      </c>
+      <c r="K15">
+        <f>K13*5</f>
+        <v>65</v>
+      </c>
+      <c r="L15" s="54">
+        <f>K15/J15</f>
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <v>44</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <v>200</v>
+      </c>
+      <c r="C17">
+        <v>85.5</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>0.42749999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>500</v>
+      </c>
+      <c r="C18">
+        <v>209</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>0.41799999999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20">
+        <v>20</v>
+      </c>
+      <c r="C20">
+        <v>6.5</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21">
+        <v>6.5</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>208</v>
+      </c>
+      <c r="B22">
+        <v>20</v>
+      </c>
+      <c r="C22">
+        <v>6.5</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>0.32500000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DF47D8-BBF7-4C16-BA97-853C39F2E503}">
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="77.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="55" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="56" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="58" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="59">
+        <v>3</v>
+      </c>
+      <c r="C5" s="56" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="58" t="s">
+        <v>217</v>
+      </c>
+      <c r="B6" s="60">
+        <v>0.04</v>
+      </c>
+      <c r="C6" s="56" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="58" t="s">
+        <v>219</v>
+      </c>
+      <c r="B7" s="60">
+        <v>0.128</v>
+      </c>
+      <c r="C7" s="56" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="58" t="s">
+        <v>221</v>
+      </c>
+      <c r="B8" s="59">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="56" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
+        <v>223</v>
+      </c>
+      <c r="B9" s="60">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="C9" s="56" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="55" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="58" t="s">
+        <v>226</v>
+      </c>
+      <c r="B12" s="61">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="58" t="s">
+        <v>227</v>
+      </c>
+      <c r="B13" s="61">
+        <v>0.38400000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="58" t="s">
+        <v>228</v>
+      </c>
+      <c r="B14" s="61">
+        <v>1.2E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="B15" s="61">
+        <v>0.81599999999999995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="58" t="s">
+        <v>230</v>
+      </c>
+      <c r="B16" s="61">
+        <v>2.1840000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="58" t="s">
+        <v>231</v>
+      </c>
+      <c r="B17" s="62">
+        <v>0.27200000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="55" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="58" t="s">
+        <v>233</v>
+      </c>
+      <c r="B20" s="63">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="58" t="s">
+        <v>234</v>
+      </c>
+      <c r="B21" s="61">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="58" t="s">
+        <v>235</v>
+      </c>
+      <c r="B22" s="61">
+        <v>8.16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="56" t="s">
+        <v>236</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E370FD39-E305-4676-A93E-6B2FD6FBE931}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="77" t="s">
+        <v>237</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="69" t="s">
+        <v>238</v>
+      </c>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="68" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="70" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="70" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="71" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" s="72">
+        <v>3</v>
+      </c>
+      <c r="C6" s="69" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="71" t="s">
+        <v>242</v>
+      </c>
+      <c r="B7" s="72">
+        <v>0.16</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="71" t="s">
+        <v>244</v>
+      </c>
+      <c r="B8" s="73">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="C8" s="69" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="71" t="s">
+        <v>246</v>
+      </c>
+      <c r="B9" s="73">
+        <v>0.04</v>
+      </c>
+      <c r="C9" s="69" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="71" t="s">
+        <v>248</v>
+      </c>
+      <c r="B10" s="72">
+        <v>0.2</v>
+      </c>
+      <c r="C10" s="67"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="71" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="73">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="C11" s="69" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="71" t="s">
+        <v>251</v>
+      </c>
+      <c r="B12" s="73">
+        <v>0.2</v>
+      </c>
+      <c r="C12" s="69" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="71" t="s">
+        <v>253</v>
+      </c>
+      <c r="B13" s="78" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="69" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="71" t="s">
+        <v>256</v>
+      </c>
+      <c r="B14" s="73">
+        <v>0.15</v>
+      </c>
+      <c r="C14" s="69" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="71" t="s">
+        <v>258</v>
+      </c>
+      <c r="B15" s="72">
+        <v>1</v>
+      </c>
+      <c r="C15" s="69" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="68" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" s="67"/>
+      <c r="C17" s="67"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="71" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" s="74">
+        <v>0.19500000000000001</v>
+      </c>
+      <c r="C18" s="67"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="71" t="s">
+        <v>262</v>
+      </c>
+      <c r="B19" s="74">
+        <v>0.32</v>
+      </c>
+      <c r="C19" s="67"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="B20" s="74">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="C20" s="67"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="71" t="s">
+        <v>264</v>
+      </c>
+      <c r="B21" s="74">
+        <v>0.68459999999999999</v>
+      </c>
+      <c r="C21" s="67"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="71" t="s">
+        <v>265</v>
+      </c>
+      <c r="B22" s="74">
+        <v>0.13691999999999999</v>
+      </c>
+      <c r="C22" s="67"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="71" t="s">
+        <v>266</v>
+      </c>
+      <c r="B23" s="74">
+        <v>0</v>
+      </c>
+      <c r="C23" s="67"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="71" t="s">
+        <v>267</v>
+      </c>
+      <c r="B24" s="74">
+        <v>0.82152000000000003</v>
+      </c>
+      <c r="C24" s="67"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="71" t="s">
+        <v>268</v>
+      </c>
+      <c r="B25" s="74">
+        <v>2.17848</v>
+      </c>
+      <c r="C25" s="67"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="71" t="s">
+        <v>269</v>
+      </c>
+      <c r="B26" s="75">
+        <v>0.27383999999999997</v>
+      </c>
+      <c r="C26" s="67"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="68" t="s">
+        <v>270</v>
+      </c>
+      <c r="B28" s="67"/>
+      <c r="C28" s="67"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="71" t="s">
+        <v>233</v>
+      </c>
+      <c r="B29" s="76">
+        <v>10</v>
+      </c>
+      <c r="C29" s="67"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="71" t="s">
+        <v>271</v>
+      </c>
+      <c r="B30" s="74">
+        <v>8.2151999999999994</v>
+      </c>
+      <c r="C30" s="67"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="71" t="s">
+        <v>272</v>
+      </c>
+      <c r="B31" s="74">
+        <v>30</v>
+      </c>
+      <c r="C31" s="69" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="69" t="s">
+        <v>274</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E308686C-2CC2-4CE9-B8BC-169E12CFA14B}">
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="89" t="s">
+        <v>275</v>
+      </c>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="81" t="s">
+        <v>276</v>
+      </c>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="80" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="82" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="82" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="82" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="83" t="s">
+        <v>215</v>
+      </c>
+      <c r="B6" s="84">
+        <v>3</v>
+      </c>
+      <c r="C6" s="81" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="83" t="s">
+        <v>278</v>
+      </c>
+      <c r="B7" s="85">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="81" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="83" t="s">
+        <v>280</v>
+      </c>
+      <c r="B8" s="84">
+        <v>0.25</v>
+      </c>
+      <c r="C8" s="81" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="83" t="s">
+        <v>282</v>
+      </c>
+      <c r="B9" s="85">
+        <v>0.02</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="83" t="s">
+        <v>284</v>
+      </c>
+      <c r="B10" s="90" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" s="81" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="83" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" s="84">
+        <v>25</v>
+      </c>
+      <c r="C11" s="79"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="83" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" s="84">
+        <v>0.75</v>
+      </c>
+      <c r="C12" s="79"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="83" t="s">
+        <v>288</v>
+      </c>
+      <c r="B13" s="85">
+        <v>0.35</v>
+      </c>
+      <c r="C13" s="81" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="80" t="s">
+        <v>290</v>
+      </c>
+      <c r="B15" s="79"/>
+      <c r="C15" s="79"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="83" t="s">
+        <v>291</v>
+      </c>
+      <c r="B16" s="86">
+        <v>0.45</v>
+      </c>
+      <c r="C16" s="79"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="83" t="s">
+        <v>292</v>
+      </c>
+      <c r="B17" s="86">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="C17" s="79"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="83" t="s">
+        <v>293</v>
+      </c>
+      <c r="B18" s="86">
+        <v>0.75</v>
+      </c>
+      <c r="C18" s="81" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="83" t="s">
+        <v>295</v>
+      </c>
+      <c r="B19" s="86">
+        <v>1.2090000000000001</v>
+      </c>
+      <c r="C19" s="79"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="83" t="s">
+        <v>296</v>
+      </c>
+      <c r="B20" s="86">
+        <v>1.7909999999999999</v>
+      </c>
+      <c r="C20" s="79"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="83" t="s">
+        <v>297</v>
+      </c>
+      <c r="B21" s="87">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="C21" s="79"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="80" t="s">
+        <v>298</v>
+      </c>
+      <c r="B23" s="79"/>
+      <c r="C23" s="79"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="83" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="88">
+        <v>10</v>
+      </c>
+      <c r="C24" s="79"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="83" t="s">
+        <v>299</v>
+      </c>
+      <c r="B25" s="86">
+        <v>12.09</v>
+      </c>
+      <c r="C25" s="79"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="83" t="s">
+        <v>300</v>
+      </c>
+      <c r="B26" s="86">
+        <v>0</v>
+      </c>
+      <c r="C26" s="79"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="83" t="s">
+        <v>301</v>
+      </c>
+      <c r="B27" s="86">
+        <v>0</v>
+      </c>
+      <c r="C27" s="81" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="81" t="s">
+        <v>303</v>
+      </c>
+      <c r="B29" s="79"/>
+      <c r="C29" s="79"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add landscape rendering functionality and associated tests
- Introduced a new script `render_landscape_sheet.py` for generating landscape bin-sticker sheets with options for style selection, all styles, and listing available styles.
- Added a comprehensive test suite in `test_render_landscape_sheet.py` to validate the functionality of the new script, including CLI argument handling and PDF generation.
- Created new icon assets for various house designs to support the rendering process.
- Updated the `StickerBinStickersCosts v2.xlsx` file with new cost data to ensure accurate pricing for the new features.

These enhancements improve the sticker generation process and ensure robust testing for the new landscape rendering capabilities.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3005BDE-59F1-4C40-B908-0B40CD916460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F018471-4EC6-4B52-9E9D-BF113DABFAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="305">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -638,9 +638,6 @@
     <t>This is now the true floor price to plan pricing around — B58/B59 above (unchanged, still used elsewhere) exclude recurring overhead entirely. The Break-Even Calculator on the Tier 1 Equipment Costs sheet pulls from B68 on this row, not from B58.</t>
   </si>
   <si>
-    <t>bank account fee</t>
-  </si>
-  <si>
     <t>full year</t>
   </si>
   <si>
@@ -951,16 +948,24 @@
   </si>
   <si>
     <t>Not wired into the 'Recurring Overhead' sheet's fixed subscription subtotal (B11) — same rationale as the eBay and Etsy blocks: variable/%-of-price costs kept separate from the flat £/sticker overhead allocation. Guide recommends holding Professional account + Sponsored Products off until Amazon volume and margin are established via eBay/Etsy first — the Y/N toggles above default to 'off' accordingly.</t>
+  </si>
+  <si>
+    <t>stikly clear</t>
+  </si>
+  <si>
+    <t>gmail account</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00000000000000"/>
+    <numFmt numFmtId="168" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="34" x14ac:knownFonts="1">
     <font>
@@ -1253,7 +1258,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1324,33 +1329,13 @@
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2198,12 +2183,12 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="64" t="s">
+      <c r="A46" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="65"/>
-      <c r="C46" s="65"/>
-      <c r="D46" s="65"/>
+      <c r="B46" s="69"/>
+      <c r="C46" s="69"/>
+      <c r="D46" s="69"/>
     </row>
     <row r="48" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="23" t="s">
@@ -2211,12 +2196,12 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="64" t="s">
+      <c r="A49" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="65"/>
-      <c r="C49" s="65"/>
-      <c r="D49" s="65"/>
+      <c r="B49" s="69"/>
+      <c r="C49" s="69"/>
+      <c r="D49" s="69"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
@@ -2235,7 +2220,7 @@
       </c>
       <c r="B52" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
-        <v>28.337866666666667</v>
+        <v>28.307866666666666</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>112</v>
@@ -2247,7 +2232,7 @@
       </c>
       <c r="B53" s="26">
         <f>B51-B52</f>
-        <v>-22.337866666666667</v>
+        <v>-22.307866666666666</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -2265,7 +2250,7 @@
       </c>
       <c r="B56" s="28">
         <f>IFERROR(B55/B53,"N/A")</f>
-        <v>-28.261875201451645</v>
+        <v>-28.299882253793879</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -2274,16 +2259,16 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
-        <v>-113.04750080580658</v>
+        <v>-113.19952901517551</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="64" t="s">
+      <c r="A59" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="B59" s="65"/>
-      <c r="C59" s="65"/>
-      <c r="D59" s="65"/>
+      <c r="B59" s="69"/>
+      <c r="C59" s="69"/>
+      <c r="D59" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2307,12 +2292,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="4" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -2395,7 +2381,7 @@
         <v>131</v>
       </c>
       <c r="B12" s="34">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="C12" s="30" t="s">
         <v>132</v>
@@ -2406,7 +2392,7 @@
         <v>133</v>
       </c>
       <c r="B13" s="34">
-        <v>0.5</v>
+        <v>0.44</v>
       </c>
       <c r="C13" s="30" t="s">
         <v>134</v>
@@ -2429,7 +2415,7 @@
       </c>
       <c r="B15" s="35">
         <f>SUM(B12:B14)</f>
-        <v>0.95000000000000007</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2447,7 +2433,7 @@
       </c>
       <c r="B18" s="35">
         <f>B15*B17</f>
-        <v>0.95000000000000007</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2549,7 +2535,7 @@
       </c>
       <c r="B30" s="40">
         <f>B18+B28</f>
-        <v>1.03</v>
+        <v>1</v>
       </c>
       <c r="C30" s="37"/>
     </row>
@@ -2559,7 +2545,7 @@
       </c>
       <c r="B31" s="42">
         <f>B30/B7</f>
-        <v>0.25750000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="C31" s="37"/>
     </row>
@@ -2616,7 +2602,7 @@
       </c>
       <c r="B37" s="40">
         <f>B36+B30</f>
-        <v>1.06</v>
+        <v>1.03</v>
       </c>
       <c r="C37" s="37"/>
     </row>
@@ -2730,19 +2716,19 @@
       </c>
       <c r="C48" s="37"/>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="37"/>
       <c r="B49" s="41"/>
       <c r="C49" s="37"/>
     </row>
-    <row r="50" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="31" t="s">
         <v>181</v>
       </c>
       <c r="B50" s="37"/>
       <c r="C50" s="37"/>
     </row>
-    <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="32" t="s">
         <v>3</v>
       </c>
@@ -2753,7 +2739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="37" t="s">
         <v>182</v>
       </c>
@@ -2764,7 +2750,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="37" t="s">
         <v>184</v>
       </c>
@@ -2773,7 +2759,7 @@
       </c>
       <c r="C53" s="37"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>185</v>
       </c>
@@ -2783,7 +2769,7 @@
       </c>
       <c r="C54" s="37"/>
     </row>
-    <row r="55" spans="1:3" ht="114.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" ht="114.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="37" t="s">
         <v>186</v>
       </c>
@@ -2794,7 +2780,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>188</v>
       </c>
@@ -2802,48 +2788,62 @@
         <f>B54/3</f>
         <v>0.21186666666666668</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D56" t="s">
+        <v>208</v>
+      </c>
+      <c r="E56" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="37"/>
       <c r="B57" s="37"/>
       <c r="C57" s="37"/>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>189</v>
       </c>
       <c r="B58" s="40">
         <f>B30+B48+B56+B36</f>
-        <v>2.1818666666666666</v>
+        <v>2.1518666666666668</v>
       </c>
       <c r="C58" s="37"/>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D58" s="66">
+        <f>B58-B12-B13+0.65</f>
+        <v>1.9318666666666671</v>
+      </c>
+      <c r="E58" s="66">
+        <f>B58-B12+0.48</f>
+        <v>2.2018666666666666</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="37" t="s">
         <v>190</v>
       </c>
       <c r="B59" s="42">
         <f>B58/B7</f>
-        <v>0.54546666666666666</v>
+        <v>0.5379666666666667</v>
       </c>
       <c r="C59" s="37"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="37"/>
       <c r="B60" s="37"/>
       <c r="C60" s="37"/>
     </row>
-    <row r="61" spans="1:3" ht="186.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" ht="186.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="39" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="31" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="32" t="s">
         <v>3</v>
       </c>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>28.337866666666667</v>
+        <v>28.307866666666666</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2890,15 +2890,15 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>7.0844666666666667</v>
+        <v>7.0769666666666664</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="66" t="s">
+      <c r="A71" s="70" t="s">
         <v>198</v>
       </c>
-      <c r="B71" s="65"/>
-      <c r="C71" s="65"/>
+      <c r="B71" s="69"/>
+      <c r="C71" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2926,12 +2926,12 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
@@ -2952,7 +2952,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3011,7 +3011,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>199</v>
+        <v>304</v>
       </c>
       <c r="B9" s="18">
         <v>10</v>
@@ -3056,12 +3056,12 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="65"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
+      <c r="B14" s="69"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
@@ -3245,47 +3245,47 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B1" t="s">
         <v>84</v>
       </c>
       <c r="C1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" t="s">
         <v>202</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>203</v>
       </c>
-      <c r="E1" t="s">
-        <v>204</v>
-      </c>
       <c r="I1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J1" t="s">
         <v>84</v>
       </c>
       <c r="K1" t="s">
+        <v>209</v>
+      </c>
+      <c r="L1" t="s">
         <v>210</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>211</v>
-      </c>
-      <c r="M1" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -3298,7 +3298,7 @@
         <v>0.65</v>
       </c>
       <c r="I3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J3">
         <v>25</v>
@@ -3314,7 +3314,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B4">
         <v>25</v>
@@ -3327,7 +3327,7 @@
         <v>0.53</v>
       </c>
       <c r="I4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J4">
         <v>50</v>
@@ -3347,7 +3347,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B5">
         <v>50</v>
@@ -3360,7 +3360,7 @@
         <v>0.45</v>
       </c>
       <c r="I5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J5">
         <v>100</v>
@@ -3380,7 +3380,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B6">
         <v>100</v>
@@ -3393,7 +3393,7 @@
         <v>0.43</v>
       </c>
       <c r="I6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J6">
         <v>200</v>
@@ -3413,7 +3413,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B7">
         <v>200</v>
@@ -3426,7 +3426,7 @@
         <v>0.4</v>
       </c>
       <c r="I7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J7">
         <v>500</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B8">
         <v>500</v>
@@ -3459,7 +3459,7 @@
         <v>0.35</v>
       </c>
       <c r="I8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J8">
         <v>25</v>
@@ -3479,7 +3479,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B9">
         <v>10</v>
@@ -3492,7 +3492,7 @@
         <v>0.75</v>
       </c>
       <c r="I9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J9">
         <v>50</v>
@@ -3522,7 +3522,7 @@
         <v>0.65</v>
       </c>
       <c r="I10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J10">
         <v>100</v>
@@ -3552,7 +3552,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="I11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J11">
         <v>200</v>
@@ -3582,7 +3582,7 @@
         <v>0.48</v>
       </c>
       <c r="I12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J12">
         <v>500</v>
@@ -3602,7 +3602,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -3615,7 +3615,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="I13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J13">
         <v>20</v>
@@ -3641,7 +3641,7 @@
         <v>0.50600000000000001</v>
       </c>
       <c r="I14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J14">
         <v>60</v>
@@ -3667,7 +3667,7 @@
         <v>0.47299999999999998</v>
       </c>
       <c r="I15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J15">
         <v>100</v>
@@ -3719,12 +3719,12 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B20">
         <v>20</v>
@@ -3739,7 +3739,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B22">
         <v>20</v>
@@ -3774,23 +3774,23 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DF47D8-BBF7-4C16-BA97-853C39F2E503}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="77.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="55" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="56" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="56" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="57" t="s">
         <v>3</v>
       </c>
@@ -3801,109 +3801,152 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="58" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B5" s="59">
         <v>3</v>
       </c>
       <c r="C5" s="56" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="58" t="s">
         <v>216</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="58" t="s">
-        <v>217</v>
       </c>
       <c r="B6" s="60">
         <v>0.04</v>
       </c>
       <c r="C6" s="56" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="58" t="s">
         <v>218</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="58" t="s">
-        <v>219</v>
       </c>
       <c r="B7" s="60">
         <v>0.128</v>
       </c>
       <c r="C7" s="56" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="58" t="s">
         <v>220</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="58" t="s">
-        <v>221</v>
       </c>
       <c r="B8" s="59">
         <v>0.3</v>
       </c>
       <c r="C8" s="56" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
         <v>222</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="58" t="s">
-        <v>223</v>
       </c>
       <c r="B9" s="60">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="C9" s="56" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="55" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="55" t="s">
+      <c r="D11">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="58" t="s">
         <v>225</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="58" t="s">
-        <v>226</v>
       </c>
       <c r="B12" s="61">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <f>B6*B5</f>
+        <v>0.12</v>
+      </c>
+      <c r="D12">
+        <f>B6*D11</f>
+        <v>0.156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B13" s="61">
         <v>0.38400000000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <f>B7*B5</f>
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="D13">
+        <f>B7*D11</f>
+        <v>0.49919999999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="58" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B14" s="61">
         <v>1.2E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C14">
+        <f>B9*B5</f>
+        <v>1.2E-2</v>
+      </c>
+      <c r="D14">
+        <f>B9*D11</f>
+        <v>1.5599999999999999E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="58" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B15" s="61">
         <v>0.81599999999999995</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C15" s="67">
+        <f>SUM(C12:C14)+B8</f>
+        <v>0.81600000000000006</v>
+      </c>
+      <c r="D15" s="67">
+        <f>SUM(D12:D14)+B8</f>
+        <v>0.97079999999999989</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B16" s="61">
         <v>2.1840000000000002</v>
       </c>
+      <c r="C16" s="67">
+        <f>B5-C15</f>
+        <v>2.1840000000000002</v>
+      </c>
+      <c r="D16" s="67">
+        <f>D11-D15</f>
+        <v>2.9291999999999998</v>
+      </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B17" s="62">
         <v>0.27200000000000002</v>
@@ -3911,12 +3954,12 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="55" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="58" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B20" s="63">
         <v>10</v>
@@ -3924,7 +3967,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B21" s="61">
         <v>1.2</v>
@@ -3932,7 +3975,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="58" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B22" s="61">
         <v>8.16</v>
@@ -3940,7 +3983,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="56" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -3952,274 +3995,255 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E370FD39-E305-4676-A93E-6B2FD6FBE931}">
   <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="64" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="56" t="s">
         <v>237</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="55" t="s">
         <v>238</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="68" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="58" t="s">
         <v>239</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="70" t="s">
+      <c r="B6" s="59">
         <v>3</v>
       </c>
-      <c r="B5" s="70" t="s">
-        <v>121</v>
-      </c>
-      <c r="C5" s="70" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="71" t="s">
+      <c r="C6" s="56" t="s">
         <v>240</v>
       </c>
-      <c r="B6" s="72">
-        <v>3</v>
-      </c>
-      <c r="C6" s="69" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="58" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="71" t="s">
+      <c r="B7" s="59">
+        <v>0.16</v>
+      </c>
+      <c r="C7" s="56" t="s">
         <v>242</v>
       </c>
-      <c r="B7" s="72">
-        <v>0.16</v>
-      </c>
-      <c r="C7" s="69" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="58" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="71" t="s">
+      <c r="B8" s="60">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="C8" s="56" t="s">
         <v>244</v>
       </c>
-      <c r="B8" s="73">
-        <v>6.5000000000000002E-2</v>
-      </c>
-      <c r="C8" s="69" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="71" t="s">
+      <c r="B9" s="60">
+        <v>0.04</v>
+      </c>
+      <c r="C9" s="56" t="s">
         <v>246</v>
       </c>
-      <c r="B9" s="73">
-        <v>0.04</v>
-      </c>
-      <c r="C9" s="69" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="58" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="71" t="s">
+      <c r="B10" s="59">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="58" t="s">
         <v>248</v>
       </c>
-      <c r="B10" s="72">
+      <c r="B11" s="60">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="C11" s="56" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="58" t="s">
+        <v>250</v>
+      </c>
+      <c r="B12" s="60">
         <v>0.2</v>
       </c>
-      <c r="C10" s="67"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="71" t="s">
-        <v>249</v>
-      </c>
-      <c r="B11" s="73">
-        <v>3.2000000000000002E-3</v>
-      </c>
-      <c r="C11" s="69" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="71" t="s">
+      <c r="C12" s="56" t="s">
         <v>251</v>
       </c>
-      <c r="B12" s="73">
-        <v>0.2</v>
-      </c>
-      <c r="C12" s="69" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="58" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="71" t="s">
+      <c r="B13" s="65" t="s">
         <v>253</v>
       </c>
-      <c r="B13" s="78" t="s">
+      <c r="C13" s="56" t="s">
         <v>254</v>
       </c>
-      <c r="C13" s="69" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="58" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="71" t="s">
+      <c r="B14" s="60">
+        <v>0.15</v>
+      </c>
+      <c r="C14" s="56" t="s">
         <v>256</v>
       </c>
-      <c r="B14" s="73">
-        <v>0.15</v>
-      </c>
-      <c r="C14" s="69" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="58" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="71" t="s">
+      <c r="B15" s="59">
+        <v>1</v>
+      </c>
+      <c r="C15" s="56" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="72">
-        <v>1</v>
-      </c>
-      <c r="C15" s="69" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="55" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="68" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="58" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="67"/>
-      <c r="C17" s="67"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="71" t="s">
+      <c r="B18" s="61">
+        <v>0.19500000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="58" t="s">
         <v>261</v>
       </c>
-      <c r="B18" s="74">
-        <v>0.19500000000000001</v>
-      </c>
-      <c r="C18" s="67"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="71" t="s">
+      <c r="B19" s="61">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="58" t="s">
         <v>262</v>
       </c>
-      <c r="B19" s="74">
-        <v>0.32</v>
-      </c>
-      <c r="C19" s="67"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="71" t="s">
+      <c r="B20" s="61">
+        <v>9.5999999999999992E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="58" t="s">
         <v>263</v>
       </c>
-      <c r="B20" s="74">
-        <v>9.5999999999999992E-3</v>
-      </c>
-      <c r="C20" s="67"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="71" t="s">
+      <c r="B21" s="61">
+        <v>0.68459999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="58" t="s">
         <v>264</v>
       </c>
-      <c r="B21" s="74">
-        <v>0.68459999999999999</v>
-      </c>
-      <c r="C21" s="67"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="71" t="s">
+      <c r="B22" s="61">
+        <v>0.13691999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="58" t="s">
         <v>265</v>
       </c>
-      <c r="B22" s="74">
-        <v>0.13691999999999999</v>
-      </c>
-      <c r="C22" s="67"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="71" t="s">
+      <c r="B23" s="61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="58" t="s">
         <v>266</v>
       </c>
-      <c r="B23" s="74">
-        <v>0</v>
-      </c>
-      <c r="C23" s="67"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="71" t="s">
+      <c r="B24" s="61">
+        <v>0.82152000000000003</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="58" t="s">
         <v>267</v>
       </c>
-      <c r="B24" s="74">
-        <v>0.82152000000000003</v>
-      </c>
-      <c r="C24" s="67"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="71" t="s">
+      <c r="B25" s="61">
+        <v>2.17848</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="58" t="s">
         <v>268</v>
       </c>
-      <c r="B25" s="74">
-        <v>2.17848</v>
-      </c>
-      <c r="C25" s="67"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="71" t="s">
+      <c r="B26" s="62">
+        <v>0.27383999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="55" t="s">
         <v>269</v>
       </c>
-      <c r="B26" s="75">
-        <v>0.27383999999999997</v>
-      </c>
-      <c r="C26" s="67"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="68" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="58" t="s">
+        <v>232</v>
+      </c>
+      <c r="B29" s="63">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="58" t="s">
         <v>270</v>
       </c>
-      <c r="B28" s="67"/>
-      <c r="C28" s="67"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="71" t="s">
-        <v>233</v>
-      </c>
-      <c r="B29" s="76">
-        <v>10</v>
-      </c>
-      <c r="C29" s="67"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="71" t="s">
+      <c r="B30" s="61">
+        <v>8.2151999999999994</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="58" t="s">
         <v>271</v>
       </c>
-      <c r="B30" s="74">
-        <v>8.2151999999999994</v>
-      </c>
-      <c r="C30" s="67"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="71" t="s">
+      <c r="B31" s="61">
+        <v>30</v>
+      </c>
+      <c r="C31" s="56" t="s">
         <v>272</v>
       </c>
-      <c r="B31" s="74">
-        <v>30</v>
-      </c>
-      <c r="C31" s="69" t="s">
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="56" t="s">
         <v>273</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="69" t="s">
-        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -4233,235 +4257,213 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="64" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="56" t="s">
         <v>275</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="81" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="55" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="58" t="s">
+        <v>214</v>
+      </c>
+      <c r="B6" s="59">
+        <v>3</v>
+      </c>
+      <c r="C6" s="56" t="s">
         <v>276</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="80" t="s">
-        <v>239</v>
-      </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="82" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="82" t="s">
-        <v>121</v>
-      </c>
-      <c r="C5" s="82" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="83" t="s">
-        <v>215</v>
-      </c>
-      <c r="B6" s="84">
-        <v>3</v>
-      </c>
-      <c r="C6" s="81" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="58" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="83" t="s">
+      <c r="B7" s="60">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="56" t="s">
         <v>278</v>
       </c>
-      <c r="B7" s="85">
-        <v>0.15</v>
-      </c>
-      <c r="C7" s="81" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="58" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="83" t="s">
+      <c r="B8" s="59">
+        <v>0.25</v>
+      </c>
+      <c r="C8" s="56" t="s">
         <v>280</v>
       </c>
-      <c r="B8" s="84">
-        <v>0.25</v>
-      </c>
-      <c r="C8" s="81" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="58" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="83" t="s">
+      <c r="B9" s="60">
+        <v>0.02</v>
+      </c>
+      <c r="C9" s="56" t="s">
         <v>282</v>
       </c>
-      <c r="B9" s="85">
-        <v>0.02</v>
-      </c>
-      <c r="C9" s="81" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="58" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="83" t="s">
+      <c r="B10" s="65" t="s">
+        <v>253</v>
+      </c>
+      <c r="C10" s="56" t="s">
         <v>284</v>
       </c>
-      <c r="B10" s="90" t="s">
-        <v>254</v>
-      </c>
-      <c r="C10" s="81" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="58" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="83" t="s">
+      <c r="B11" s="59">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="58" t="s">
         <v>286</v>
       </c>
-      <c r="B11" s="84">
-        <v>25</v>
-      </c>
-      <c r="C11" s="79"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="83" t="s">
+      <c r="B12" s="59">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="58" t="s">
         <v>287</v>
       </c>
-      <c r="B12" s="84">
+      <c r="B13" s="60">
+        <v>0.35</v>
+      </c>
+      <c r="C13" s="56" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="55" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="58" t="s">
+        <v>290</v>
+      </c>
+      <c r="B16" s="61">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="58" t="s">
+        <v>291</v>
+      </c>
+      <c r="B17" s="61">
+        <v>0.45900000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="58" t="s">
+        <v>292</v>
+      </c>
+      <c r="B18" s="61">
         <v>0.75</v>
       </c>
-      <c r="C12" s="79"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="83" t="s">
-        <v>288</v>
-      </c>
-      <c r="B13" s="85">
-        <v>0.35</v>
-      </c>
-      <c r="C13" s="81" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="80" t="s">
-        <v>290</v>
-      </c>
-      <c r="B15" s="79"/>
-      <c r="C15" s="79"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="83" t="s">
-        <v>291</v>
-      </c>
-      <c r="B16" s="86">
-        <v>0.45</v>
-      </c>
-      <c r="C16" s="79"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="83" t="s">
-        <v>292</v>
-      </c>
-      <c r="B17" s="86">
-        <v>0.45900000000000002</v>
-      </c>
-      <c r="C17" s="79"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="83" t="s">
+      <c r="C18" s="56" t="s">
         <v>293</v>
       </c>
-      <c r="B18" s="86">
-        <v>0.75</v>
-      </c>
-      <c r="C18" s="81" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="58" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="83" t="s">
+      <c r="B19" s="61">
+        <v>1.2090000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="58" t="s">
         <v>295</v>
       </c>
-      <c r="B19" s="86">
-        <v>1.2090000000000001</v>
-      </c>
-      <c r="C19" s="79"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="83" t="s">
+      <c r="B20" s="61">
+        <v>1.7909999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="58" t="s">
         <v>296</v>
       </c>
-      <c r="B20" s="86">
-        <v>1.7909999999999999</v>
-      </c>
-      <c r="C20" s="79"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="83" t="s">
+      <c r="B21" s="62">
+        <v>0.40300000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="55" t="s">
         <v>297</v>
       </c>
-      <c r="B21" s="87">
-        <v>0.40300000000000002</v>
-      </c>
-      <c r="C21" s="79"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="80" t="s">
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="58" t="s">
+        <v>232</v>
+      </c>
+      <c r="B24" s="63">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="58" t="s">
         <v>298</v>
       </c>
-      <c r="B23" s="79"/>
-      <c r="C23" s="79"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="83" t="s">
-        <v>233</v>
-      </c>
-      <c r="B24" s="88">
-        <v>10</v>
-      </c>
-      <c r="C24" s="79"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="83" t="s">
+      <c r="B25" s="61">
+        <v>12.09</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="58" t="s">
         <v>299</v>
       </c>
-      <c r="B25" s="86">
-        <v>12.09</v>
-      </c>
-      <c r="C25" s="79"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="83" t="s">
+      <c r="B26" s="61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="58" t="s">
         <v>300</v>
       </c>
-      <c r="B26" s="86">
+      <c r="B27" s="61">
         <v>0</v>
       </c>
-      <c r="C26" s="79"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="83" t="s">
+      <c r="C27" s="56" t="s">
         <v>301</v>
       </c>
-      <c r="B27" s="86">
-        <v>0</v>
-      </c>
-      <c r="C27" s="81" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="56" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="81" t="s">
-        <v>303</v>
-      </c>
-      <c r="B29" s="79"/>
-      <c r="C29" s="79"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Implement updates for Platform Selling Fees and Analytics Dashboard
- Added new files for the Platform Selling Fees and Analytics Dashboard features, including detailed specifications and data model changes.
- Introduced new tables for tracking platform fees and recurring expenses, enhancing the plugin's financial tracking capabilities.
- Developed a new cron job for syncing platform fees from eBay and Etsy APIs, ensuring accurate fee data is captured.
- Created an Analytics Dashboard with visualizations for sales, profit, and material stock over time, utilizing Chart.js for dynamic charting.
- Updated the sprint plan to outline implementation steps and open items for further development.

These enhancements significantly improve the plugin's functionality, providing users with better insights into their sales and associated costs.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F018471-4EC6-4B52-9E9D-BF113DABFAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DDA96A-014D-4735-B6AB-C5D390F52D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="306">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -954,6 +954,9 @@
   </si>
   <si>
     <t>gmail account</t>
+  </si>
+  <si>
+    <t>domain</t>
   </si>
 </sst>
 </file>
@@ -2220,7 +2223,7 @@
       </c>
       <c r="B52" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
-        <v>28.307866666666666</v>
+        <v>29.027866666666664</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>112</v>
@@ -2232,7 +2235,7 @@
       </c>
       <c r="B53" s="26">
         <f>B51-B52</f>
-        <v>-22.307866666666666</v>
+        <v>-23.027866666666664</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -2250,7 +2253,7 @@
       </c>
       <c r="B56" s="28">
         <f>IFERROR(B55/B53,"N/A")</f>
-        <v>-28.299882253793879</v>
+        <v>-27.415044960019454</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -2259,7 +2262,7 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
-        <v>-113.19952901517551</v>
+        <v>-109.66017984007782</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -2859,8 +2862,8 @@
         <v>193</v>
       </c>
       <c r="B65" s="43">
-        <f>'Recurring Overhead'!B33</f>
-        <v>6.5389999999999997</v>
+        <f>'Recurring Overhead'!B34</f>
+        <v>6.7189999999999994</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>194</v>
@@ -2872,7 +2875,7 @@
       </c>
       <c r="B66" s="41">
         <f>B65*B7</f>
-        <v>26.155999999999999</v>
+        <v>26.875999999999998</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -2881,7 +2884,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>28.307866666666666</v>
+        <v>29.027866666666664</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2890,7 +2893,7 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>7.0769666666666664</v>
+        <v>7.2569666666666661</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -2911,7 +2914,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -3011,219 +3014,230 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>304</v>
-      </c>
-      <c r="B9" s="18">
-        <v>10</v>
-      </c>
+        <v>305</v>
+      </c>
+      <c r="B9" s="18"/>
       <c r="C9" s="17"/>
       <c r="D9" s="1"/>
       <c r="E9">
-        <f>B9*12</f>
-        <v>120</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B10" s="18">
+        <v>11.8</v>
+      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="1"/>
+      <c r="E10">
+        <f>B10*12</f>
+        <v>141.60000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B11" s="18">
         <v>0</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C11" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="20">
-        <f>SUM(B6:B10)</f>
-        <v>65.39</v>
-      </c>
-      <c r="E11">
-        <f>SUM(E6:E10)</f>
-        <v>646.74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="B12" s="20">
+        <f>SUM(B6:B11)</f>
+        <v>67.19</v>
+      </c>
+      <c r="E12">
+        <f>SUM(E6:E11)</f>
+        <v>698.34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="68" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
-      <c r="D14" s="69"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="16" t="s">
+      <c r="B15" s="69"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B17" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C17" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D17" s="16" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="44">
-        <v>10</v>
-      </c>
-      <c r="C17" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B18" s="44">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="44">
+        <v>40</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="45">
-        <f>B21</f>
+      <c r="B20" s="45">
+        <f>B22</f>
         <v>1</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C20" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="46">
-        <v>1</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="46">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="45">
-        <f>IFERROR(B21*4.33/(45/60)*20,0)</f>
+      <c r="B23" s="45">
+        <f>IFERROR(B22*4.33/(45/60)*20,0)</f>
         <v>115.46666666666667</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B26" s="16" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B26" s="27">
-        <f>IFERROR($B$11/B17,0)</f>
-        <v>6.5389999999999997</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B27" s="27">
-        <f>IFERROR($B$11/B18,0)</f>
-        <v>1.6347499999999999</v>
+        <f>IFERROR($B$12/B18,0)</f>
+        <v>6.7189999999999994</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="27">
+        <f>IFERROR($B$12/B19,0)</f>
+        <v>1.6797499999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="27">
-        <f>IFERROR($B$11/B19,0)</f>
-        <v>65.39</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="B29" s="27">
+        <f>IFERROR($B$12/B20,0)</f>
+        <v>67.19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="45">
-        <f>INDEX(B17:B19,MATCH(B31,A17:A19,0))</f>
+      <c r="B33" s="45">
+        <f>INDEX(B18:B20,MATCH(B32,A18:A20,0))</f>
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="19" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="20">
-        <f>IFERROR($B$11/B32,0)</f>
-        <v>6.5389999999999997</v>
+      <c r="B34" s="20">
+        <f>IFERROR($B$12/B33,0)</f>
+        <v>6.7189999999999994</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="B31" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="B32" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Conservative,Base / Target,Optimistic / Capacity ceiling"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Update sticker design files and expand product gallery
- Updated the `bin_sticker_products_gallery_data.md` and `bin_sticker_products_gallery.html` to reflect a total of 23 catalogued entries, increasing from 17.
- Added new designs for wreath-themed stickers (D18 to D23) with detailed descriptions and marketing angles.
- Introduced new icon assets for various wreath designs, enhancing the visual representation of the product offerings.
- Fixed a bug in the text drawing function to allow for proper rotation based on curve coefficients, improving the rendering of curved text in designs.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DDA96A-014D-4735-B6AB-C5D390F52D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C11E69F-966A-4841-B5E8-CC75F5E9E884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -1908,7 +1908,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="50" t="s">
+      <c r="A31" s="49" t="s">
         <v>85</v>
       </c>
       <c r="B31" s="18">
@@ -1928,7 +1928,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="50" t="s">
+      <c r="A32" s="49" t="s">
         <v>87</v>
       </c>
       <c r="B32" s="18">

</xml_diff>

<commit_message>
Revise sticker business plan and update cost estimates
- Adjusted the total startup cost for sticker production, reflecting changes in required equipment and materials.
- Updated packaging details for bin stickers, including size reduction and cost implications.
- Clarified production steps for sticker creation, emphasizing the use of Cricut's Print-Then-Cut feature.
- Noted unresolved questions regarding multi-item order packaging strategies.

This update aims to provide clearer guidance on costs and production methods for the sticker business.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C11E69F-966A-4841-B5E8-CC75F5E9E884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE677F76-7DB4-49C2-B0B1-219A067453E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Enhance sticker layout functionality and add new test files
- Introduced dynamic font sizing for house numbers in `bin_sticker.py` to ensure proper rendering across varying lengths.
- Added a new constant for asymmetric margins in landscape layouts, improving print alignment.
- Created `render_flourish_layout_sheet.py` for generating layout tests with various house number and street name combinations.
- Added two new PDF files (`flourish_layout_test.pdf` and `landscape_all.pdf`) to visualize layout outputs for testing purposes.
- Updated `StickerBinStickersCosts v2.xlsx` to reflect changes in layout design considerations.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE677F76-7DB4-49C2-B0B1-219A067453E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C17319A-4702-4D2D-956F-734622592004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="307">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -957,6 +957,9 @@
   </si>
   <si>
     <t>domain</t>
+  </si>
+  <si>
+    <t>210 x 297mm Rectangle, Avery Blank Labels | Avery</t>
   </si>
 </sst>
 </file>
@@ -1604,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2168,116 +2171,124 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="19" t="s">
+      <c r="A43" s="51" t="s">
+        <v>306</v>
+      </c>
+      <c r="B43" s="18"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="1"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="20">
+      <c r="B44" s="20">
         <f>SUM(B31:B42)</f>
         <v>102.31</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="21" t="s">
+    <row r="46" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="B45" s="22">
-        <f>B14+B43</f>
+      <c r="B46" s="22">
+        <f>B14+B44</f>
         <v>631.30999999999995</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="68" t="s">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="69"/>
-      <c r="C46" s="69"/>
-      <c r="D46" s="69"/>
-    </row>
-    <row r="48" spans="1:9" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="23" t="s">
+      <c r="B47" s="69"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="69"/>
+    </row>
+    <row r="49" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="68" t="s">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="B49" s="69"/>
-      <c r="C49" s="69"/>
-      <c r="D49" s="69"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="B51" s="18">
-        <v>6</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>110</v>
-      </c>
+      <c r="B50" s="69"/>
+      <c r="C50" s="69"/>
+      <c r="D50" s="69"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="B52" s="18">
+        <v>6</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="B52" s="24">
+      <c r="B53" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
         <v>29.027866666666664</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="25" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="B53" s="26">
-        <f>B51-B52</f>
+      <c r="B54" s="26">
+        <f>B52-B53</f>
         <v>-23.027866666666664</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="17" t="s">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="B55" s="27">
-        <f>B45</f>
+      <c r="B56" s="27">
+        <f>B46</f>
         <v>631.30999999999995</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="B56" s="28">
-        <f>IFERROR(B55/B53,"N/A")</f>
-        <v>-27.415044960019454</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B57" s="28">
+        <f>IFERROR(B56/B54,"N/A")</f>
+        <v>-27.415044960019454</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B57" s="28">
-        <f>IFERROR(B56*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
+      <c r="B58" s="28">
+        <f>IFERROR(B57*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
         <v>-109.66017984007782</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="68" t="s">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="B59" s="69"/>
-      <c r="C59" s="69"/>
-      <c r="D59" s="69"/>
+      <c r="B60" s="69"/>
+      <c r="C60" s="69"/>
+      <c r="D60" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A34" r:id="rId1" display="https://www.amazon.co.uk/dp/B0DK3V552G?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -2287,6 +2298,7 @@
     <hyperlink ref="A38" r:id="rId5" display="https://www.amazon.co.uk/dp/B0BNQW8LY3?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="A39" r:id="rId6" display="https://www.amazon.co.uk/dp/B0DFZ6585M?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="A40" r:id="rId7" display="https://www.amazon.co.uk/dp/B094454Q6P?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="A43" r:id="rId8" display="https://www.avery.co.uk/blank-labels/rectangle-210x297mm?mat=wop" xr:uid="{E3D54250-8282-46DF-B69A-4347BD41481B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update Excel files for sticker costs and test tracking
- Modified `StickerBinStickersCosts v2.xlsx` to reflect updated cost estimates and layout considerations for sticker production.
- Updated `Test-Tracking-Sheet.xlsx` to enhance tracking capabilities for testing processes and results.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C17319A-4702-4D2D-956F-734622592004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76B0ED2-CE7D-4B78-BC2A-58572628FF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="307">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -1607,7 +1607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B53" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
-        <v>29.027866666666664</v>
+        <v>29.075999999999997</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>112</v>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B54" s="26">
         <f>B52-B53</f>
-        <v>-23.027866666666664</v>
+        <v>-23.075999999999997</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56/B54,"N/A")</f>
-        <v>-27.415044960019454</v>
+        <v>-27.357860981105912</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B58" s="28">
         <f>IFERROR(B57*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
-        <v>-109.66017984007782</v>
+        <v>-109.43144392442365</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -2283,6 +2283,11 @@
       <c r="B60" s="69"/>
       <c r="C60" s="69"/>
       <c r="D60" s="69"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="51" t="s">
+        <v>306</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2299,6 +2304,7 @@
     <hyperlink ref="A39" r:id="rId6" display="https://www.amazon.co.uk/dp/B0DFZ6585M?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="A40" r:id="rId7" display="https://www.amazon.co.uk/dp/B094454Q6P?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="A43" r:id="rId8" display="https://www.avery.co.uk/blank-labels/rectangle-210x297mm?mat=wop" xr:uid="{E3D54250-8282-46DF-B69A-4347BD41481B}"/>
+    <hyperlink ref="A64" r:id="rId9" display="https://www.avery.co.uk/blank-labels/rectangle-210x297mm?mat=wop" xr:uid="{85EB6DCF-BF48-4CCD-99E1-16242BE1FA3E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2396,7 +2402,7 @@
         <v>131</v>
       </c>
       <c r="B12" s="34">
-        <v>0.43</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="C12" s="30" t="s">
         <v>132</v>
@@ -2407,7 +2413,7 @@
         <v>133</v>
       </c>
       <c r="B13" s="34">
-        <v>0.44</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="C13" s="30" t="s">
         <v>134</v>
@@ -2430,7 +2436,7 @@
       </c>
       <c r="B15" s="35">
         <f>SUM(B12:B14)</f>
-        <v>0.92</v>
+        <v>0.70000000000000007</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2448,7 +2454,7 @@
       </c>
       <c r="B18" s="35">
         <f>B15*B17</f>
-        <v>0.92</v>
+        <v>0.70000000000000007</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2550,7 +2556,7 @@
       </c>
       <c r="B30" s="40">
         <f>B18+B28</f>
-        <v>1</v>
+        <v>0.78</v>
       </c>
       <c r="C30" s="37"/>
     </row>
@@ -2560,7 +2566,7 @@
       </c>
       <c r="B31" s="42">
         <f>B30/B7</f>
-        <v>0.25</v>
+        <v>0.19500000000000001</v>
       </c>
       <c r="C31" s="37"/>
     </row>
@@ -2596,7 +2602,7 @@
         <v>159</v>
       </c>
       <c r="B35">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="C35" t="s">
         <v>160</v>
@@ -2608,7 +2614,7 @@
       </c>
       <c r="B36">
         <f>SUM(B34:B35)</f>
-        <v>0.03</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2617,7 +2623,7 @@
       </c>
       <c r="B37" s="40">
         <f>B36+B30</f>
-        <v>1.03</v>
+        <v>0.85000000000000009</v>
       </c>
       <c r="C37" s="37"/>
     </row>
@@ -2759,7 +2765,7 @@
         <v>182</v>
       </c>
       <c r="B52" s="34">
-        <v>15.89</v>
+        <v>33</v>
       </c>
       <c r="C52" s="39" t="s">
         <v>183</v>
@@ -2780,7 +2786,7 @@
       </c>
       <c r="B54" s="40">
         <f>B52/B53</f>
-        <v>0.63560000000000005</v>
+        <v>1.32</v>
       </c>
       <c r="C54" s="37"/>
     </row>
@@ -2801,7 +2807,7 @@
       </c>
       <c r="B56">
         <f>B54/3</f>
-        <v>0.21186666666666668</v>
+        <v>0.44</v>
       </c>
       <c r="D56" t="s">
         <v>208</v>
@@ -2821,16 +2827,16 @@
       </c>
       <c r="B58" s="40">
         <f>B30+B48+B56+B36</f>
-        <v>2.1518666666666668</v>
+        <v>2.1999999999999997</v>
       </c>
       <c r="C58" s="37"/>
       <c r="D58" s="66">
         <f>B58-B12-B13+0.65</f>
-        <v>1.9318666666666671</v>
+        <v>2.1999999999999997</v>
       </c>
       <c r="E58" s="66">
         <f>B58-B12+0.48</f>
-        <v>2.2018666666666666</v>
+        <v>2.3549999999999995</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
@@ -2839,7 +2845,7 @@
       </c>
       <c r="B59" s="42">
         <f>B58/B7</f>
-        <v>0.5379666666666667</v>
+        <v>0.54999999999999993</v>
       </c>
       <c r="C59" s="37"/>
     </row>
@@ -2896,7 +2902,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>29.027866666666664</v>
+        <v>29.075999999999997</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2905,7 +2911,7 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>7.2569666666666661</v>
+        <v>7.2689999999999992</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -3800,23 +3806,23 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DF47D8-BBF7-4C16-BA97-853C39F2E503}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="77.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="55" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="56" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="57" t="s">
         <v>3</v>
       </c>
@@ -3827,18 +3833,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="58" t="s">
         <v>214</v>
       </c>
       <c r="B5" s="59">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="C5" s="56" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="58" t="s">
         <v>216</v>
       </c>
@@ -3849,7 +3855,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="58" t="s">
         <v>218</v>
       </c>
@@ -3860,7 +3866,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="58" t="s">
         <v>220</v>
       </c>
@@ -3871,7 +3877,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="58" t="s">
         <v>222</v>
       </c>
@@ -3882,15 +3888,18 @@
         <v>223</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="55" t="s">
         <v>224</v>
       </c>
       <c r="D11">
         <v>3.9</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="58" t="s">
         <v>225</v>
       </c>
@@ -3899,14 +3908,18 @@
       </c>
       <c r="C12">
         <f>B6*B5</f>
-        <v>0.12</v>
+        <v>0.12400000000000001</v>
       </c>
       <c r="D12">
         <f>B6*D11</f>
         <v>0.156</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12">
+        <f>B6*E11</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="58" t="s">
         <v>226</v>
       </c>
@@ -3915,14 +3928,18 @@
       </c>
       <c r="C13">
         <f>B7*B5</f>
-        <v>0.38400000000000001</v>
+        <v>0.39680000000000004</v>
       </c>
       <c r="D13">
         <f>B7*D11</f>
         <v>0.49919999999999998</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13">
+        <f>B7*E11</f>
+        <v>0.51200000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="58" t="s">
         <v>227</v>
       </c>
@@ -3931,14 +3948,18 @@
       </c>
       <c r="C14">
         <f>B9*B5</f>
-        <v>1.2E-2</v>
+        <v>1.2400000000000001E-2</v>
       </c>
       <c r="D14">
         <f>B9*D11</f>
         <v>1.5599999999999999E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14">
+        <f>B8*E13</f>
+        <v>0.15359999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="58" t="s">
         <v>228</v>
       </c>
@@ -3947,14 +3968,18 @@
       </c>
       <c r="C15" s="67">
         <f>SUM(C12:C14)+B8</f>
-        <v>0.81600000000000006</v>
+        <v>0.83319999999999994</v>
       </c>
       <c r="D15" s="67">
         <f>SUM(D12:D14)+B8</f>
         <v>0.97079999999999989</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E15">
+        <f t="shared" ref="E13:E16" si="0">B9*E14</f>
+        <v>6.1439999999999997E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="58" t="s">
         <v>229</v>
       </c>
@@ -3963,11 +3988,15 @@
       </c>
       <c r="C16" s="67">
         <f>B5-C15</f>
-        <v>2.1840000000000002</v>
+        <v>2.2667999999999999</v>
       </c>
       <c r="D16" s="67">
         <f>D11-D15</f>
         <v>2.9291999999999998</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add new design PDF and update sticker costs file
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76B0ED2-CE7D-4B78-BC2A-58572628FF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9674F21-5146-47DD-ACEE-751FDD56EB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Amazon" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="313">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -960,6 +961,24 @@
   </si>
   <si>
     <t>210 x 297mm Rectangle, Avery Blank Labels | Avery</t>
+  </si>
+  <si>
+    <t>virtual office</t>
+  </si>
+  <si>
+    <t>https://cricut.com/en-gb/cutting-machines/cricut-joy/cricut-joy-xtra</t>
+  </si>
+  <si>
+    <t>lamp</t>
+  </si>
+  <si>
+    <t>bin</t>
+  </si>
+  <si>
+    <t>tools</t>
+  </si>
+  <si>
+    <t>Desktop File Holder A4 Paper Storage Letter Tray Office Document Sort Organiser | eBay UK</t>
   </si>
 </sst>
 </file>
@@ -1607,7 +1626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -2287,6 +2306,52 @@
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="51" t="s">
         <v>306</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>308</v>
+      </c>
+      <c r="B65">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>309</v>
+      </c>
+      <c r="B66">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>310</v>
+      </c>
+      <c r="B67">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>311</v>
+      </c>
+      <c r="B68">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="51" t="s">
+        <v>312</v>
+      </c>
+      <c r="B69">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B70">
+        <f>SUM(B65:B69)</f>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2305,6 +2370,7 @@
     <hyperlink ref="A40" r:id="rId7" display="https://www.amazon.co.uk/dp/B094454Q6P?ref=ppx_yo2ov_dt_b_fed_asin_title" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="A43" r:id="rId8" display="https://www.avery.co.uk/blank-labels/rectangle-210x297mm?mat=wop" xr:uid="{E3D54250-8282-46DF-B69A-4347BD41481B}"/>
     <hyperlink ref="A64" r:id="rId9" display="https://www.avery.co.uk/blank-labels/rectangle-210x297mm?mat=wop" xr:uid="{85EB6DCF-BF48-4CCD-99E1-16242BE1FA3E}"/>
+    <hyperlink ref="A69" r:id="rId10" display="https://www.ebay.co.uk/itm/298422348734" xr:uid="{7322324D-F8B7-4017-ACB0-DA34DF58D45B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2880,7 +2946,7 @@
         <v>193</v>
       </c>
       <c r="B65" s="43">
-        <f>'Recurring Overhead'!B34</f>
+        <f>'Recurring Overhead'!B35</f>
         <v>6.7189999999999994</v>
       </c>
       <c r="C65" s="2" t="s">
@@ -2932,7 +2998,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -3070,192 +3136,203 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="1"/>
+      <c r="E12">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B13" s="20">
         <f>SUM(B6:B11)</f>
         <v>67.19</v>
       </c>
-      <c r="E12">
-        <f>SUM(E6:E11)</f>
-        <v>698.34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="E13">
+        <f>SUM(E6:E12)</f>
+        <v>948.34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="68" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="69"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B18" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C18" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D18" s="16" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="44">
-        <v>10</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B19" s="44">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="44">
+        <v>40</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="45">
-        <f>B22</f>
+      <c r="B21" s="45">
+        <f>B23</f>
         <v>1</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C21" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="46">
-        <v>1</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="46">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="45">
-        <f>IFERROR(B22*4.33/(45/60)*20,0)</f>
+      <c r="B24" s="45">
+        <f>IFERROR(B23*4.33/(45/60)*20,0)</f>
         <v>115.46666666666667</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="16" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B27" s="16" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="27">
-        <f>IFERROR($B$12/B18,0)</f>
-        <v>6.7189999999999994</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B28" s="27">
-        <f>IFERROR($B$12/B19,0)</f>
-        <v>1.6797499999999999</v>
+        <f>IFERROR($B$13/B19,0)</f>
+        <v>6.7189999999999994</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="27">
+        <f>IFERROR($B$13/B20,0)</f>
+        <v>1.6797499999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="27">
-        <f>IFERROR($B$12/B20,0)</f>
+      <c r="B30" s="27">
+        <f>IFERROR($B$13/B21,0)</f>
         <v>67.19</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="17" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B32" s="47" t="s">
+      <c r="B33" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B33" s="45">
-        <f>INDEX(B18:B20,MATCH(B32,A18:A20,0))</f>
+      <c r="B34" s="45">
+        <f>INDEX(B19:B21,MATCH(B33,A19:A21,0))</f>
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="19" t="s">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="20">
-        <f>IFERROR($B$12/B33,0)</f>
+      <c r="B35" s="20">
+        <f>IFERROR($B$13/B34,0)</f>
         <v>6.7189999999999994</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="B32" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="B33" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Conservative,Base / Target,Optimistic / Capacity ceiling"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3975,7 +4052,7 @@
         <v>0.97079999999999989</v>
       </c>
       <c r="E15">
-        <f t="shared" ref="E13:E16" si="0">B9*E14</f>
+        <f>B9*E14</f>
         <v>6.1439999999999997E-4</v>
       </c>
     </row>
@@ -3995,7 +4072,7 @@
         <v>2.9291999999999998</v>
       </c>
       <c r="E16">
-        <f t="shared" si="0"/>
+        <f>B10*E15</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>